<commit_message>
feat: add 'Exporteer inkoopvoorstel' button with Excel enrichment export
</commit_message>
<xml_diff>
--- a/public/sjabloon-valuetracker-overtollige-artikelen-parttracker.xlsx
+++ b/public/sjabloon-valuetracker-overtollige-artikelen-parttracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29816"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29905"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://parttrackereu-my.sharepoint.com/personal/alex_parttracker_eu/Documents/PARTTRACKER 2026/Voorraad/Overtollige voorraad/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{985C07F3-82EC-47BB-8A12-816DC975D9B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{48390E0B-9468-4545-917E-9BE33CCA979A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="165" windowWidth="42480" windowHeight="15435" xr2:uid="{A0943E84-8AC0-4323-AF99-BA9B0E589237}"/>
+    <workbookView xWindow="1155" yWindow="420" windowWidth="30540" windowHeight="15165" xr2:uid="{A0943E84-8AC0-4323-AF99-BA9B0E589237}"/>
   </bookViews>
   <sheets>
     <sheet name="Artikel lijst" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="45">
   <si>
     <t xml:space="preserve">OEV lijst voor verkoop via PartTracker </t>
   </si>
@@ -48,9 +48,6 @@
   </si>
   <si>
     <t>Uitleg over dit document vindt u in de tab "werkwijze" of klik hier</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Datum verzending: </t>
   </si>
   <si>
     <t>Locaties:</t>
@@ -62,7 +59,7 @@
     <t>Regel</t>
   </si>
   <si>
-    <t>Locatie*</t>
+    <t>Locatie</t>
   </si>
   <si>
     <t>Fabrikant*</t>
@@ -77,7 +74,7 @@
     <t>Bestelnummer fabrikant</t>
   </si>
   <si>
-    <t>Categorie</t>
+    <t>Categorie*</t>
   </si>
   <si>
     <t xml:space="preserve">Aantal* </t>
@@ -86,19 +83,16 @@
     <t>Eenheid*</t>
   </si>
   <si>
-    <t>Conditie</t>
+    <t>Conditie*</t>
   </si>
   <si>
-    <t>Datum*</t>
+    <t>Aankoop datum</t>
   </si>
   <si>
-    <t>Bruto Prijs p.st*</t>
+    <t>Bruto Prijs fabrikant</t>
   </si>
   <si>
-    <t>Totaal</t>
-  </si>
-  <si>
-    <t>St</t>
+    <t>Waarde p/st (in vullen door PartTracker)</t>
   </si>
   <si>
     <t>* = verplichte velden</t>
@@ -126,6 +120,9 @@
   </si>
   <si>
     <t>betreft gebruikt artikel,(gebruikssporen, werkend artikel, met functionerings garantie vanuit de aanbieder)</t>
+  </si>
+  <si>
+    <t>Categorie</t>
   </si>
   <si>
     <t>Frequentie regelaars</t>
@@ -184,9 +181,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="44" formatCode="_ &quot;€&quot;\ * #,##0.00_ ;_ &quot;€&quot;\ * \-#,##0.00_ ;_ &quot;€&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="164" formatCode="_ &quot;€&quot;\ * #,##0.00_ ;_ &quot;€&quot;\ * \-#,##0.00_ ;_ &quot;€&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -260,8 +257,16 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -297,8 +302,14 @@
         <fgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7030A0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="24">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -343,19 +354,6 @@
         <color indexed="64"/>
       </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -605,71 +603,119 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="44" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="17" fontId="5" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="17" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="9" xfId="5" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="10" fillId="5" borderId="1" xfId="5" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="9" fillId="0" borderId="9" xfId="5" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="10" fillId="5" borderId="11" xfId="5" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="17" fontId="5" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="17" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="5" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="5" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="8" xfId="5" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="10" xfId="5" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="11" fillId="7" borderId="8" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="23" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="24" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="25" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -703,168 +749,10 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>190499</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>238125</xdr:colOff>
-      <xdr:row>16</xdr:row>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>34399</xdr:colOff>
+      <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="Tekstvak 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1D0A23E8-999F-4265-B739-EF25DFE33A67}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="14706600" y="1933574"/>
-          <a:ext cx="2781300" cy="1209676"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:solidFill>
-            <a:schemeClr val="lt1">
-              <a:shade val="50000"/>
-            </a:schemeClr>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:r>
-            <a:rPr lang="nl-NL" sz="1200" b="1">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Service</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="nl-NL" sz="1200" b="1" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> en contact:</a:t>
-          </a:r>
-          <a:endParaRPr lang="nl-NL" sz="1200" b="1">
-            <a:solidFill>
-              <a:schemeClr val="tx1"/>
-            </a:solidFill>
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="nl-NL" sz="1200" b="1">
-              <a:solidFill>
-                <a:srgbClr val="7030A0"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>PartTracke</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="nl-NL" sz="1200" b="1" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="7030A0"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>r BV.</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="nl-NL" sz="1200" baseline="0">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Tel:  +31 (0)85-0708222</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="nl-NL" sz="1200" baseline="0">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>sales@parttracker.eu</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="nl-NL" sz="1200" baseline="0">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>www.parttracker.eu</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:br>
-            <a:rPr lang="nl-NL" sz="1200" baseline="0">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-          </a:br>
-          <a:endParaRPr lang="nl-NL" sz="1200" baseline="0">
-            <a:solidFill>
-              <a:schemeClr val="dk1"/>
-            </a:solidFill>
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:ea typeface="+mn-ea"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>72499</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>57154</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
@@ -885,10 +773,10 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="72499" y="57154"/>
-          <a:ext cx="12336672" cy="1390647"/>
-          <a:chOff x="55177" y="10334625"/>
-          <a:chExt cx="9388875" cy="1422206"/>
+          <a:off x="34399" y="0"/>
+          <a:ext cx="12374772" cy="1447801"/>
+          <a:chOff x="26181" y="10276174"/>
+          <a:chExt cx="9417871" cy="1480657"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:pic>
@@ -912,8 +800,8 @@
         </xdr:blipFill>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="55177" y="10354103"/>
-            <a:ext cx="910430" cy="1285833"/>
+            <a:off x="26181" y="10276174"/>
+            <a:ext cx="756717" cy="1363762"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -1180,22 +1068,171 @@
               <a:ea typeface="Aptos" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
             </a:rPr>
-            <a:t>Versie: 4, augustus 2025</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="nl-NL" sz="1100" b="1" kern="100">
-              <a:effectLst/>
-              <a:latin typeface="Aptos" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Aptos" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-            </a:rPr>
-            <a:t>.</a:t>
+            <a:t>Versie: 5, Maart 2026</a:t>
           </a:r>
           <a:endParaRPr lang="nl-NL" sz="1100" kern="100">
             <a:effectLst/>
             <a:latin typeface="Aptos" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
             <a:ea typeface="Aptos" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
             <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>180974</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>1162050</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="Tekstvak 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1D0A23E8-999F-4265-B739-EF25DFE33A67}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9505950" y="752474"/>
+          <a:ext cx="2647950" cy="1104901"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="nl-NL" sz="1200" b="1">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>Service</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="nl-NL" sz="1200" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t> en contact:</a:t>
+          </a:r>
+          <a:endParaRPr lang="nl-NL" sz="1200" b="1">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="nl-NL" sz="1200" b="1">
+              <a:solidFill>
+                <a:srgbClr val="7030A0"/>
+              </a:solidFill>
+              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>PartTracke</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="nl-NL" sz="1200" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="7030A0"/>
+              </a:solidFill>
+              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>r BV.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="nl-NL" sz="1200" baseline="0">
+              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>Tel:  +31 (0)85-0708222</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="nl-NL" sz="1200" baseline="0">
+              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>sales@parttracker.eu</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="nl-NL" sz="1200" baseline="0">
+              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>www.parttracker.eu</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:br>
+            <a:rPr lang="nl-NL" sz="1200" baseline="0">
+              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+          </a:br>
+          <a:endParaRPr lang="nl-NL" sz="1200" baseline="0">
+            <a:solidFill>
+              <a:schemeClr val="dk1"/>
+            </a:solidFill>
+            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
           </a:endParaRPr>
         </a:p>
       </xdr:txBody>
@@ -1839,7 +1876,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>enheid:</a:t>
+            <a:t>Eenheid:</a:t>
           </a:r>
           <a:br>
             <a:rPr lang="nl-NL" sz="1100" b="0" baseline="0">
@@ -3046,9 +3083,9 @@
     <col min="7" max="7" width="17" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="11.140625" customWidth="1"/>
     <col min="10" max="10" width="19.140625" customWidth="1"/>
-    <col min="11" max="11" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.5703125" customWidth="1"/>
     <col min="12" max="12" width="15.140625" customWidth="1"/>
-    <col min="13" max="13" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="27.85546875" customWidth="1"/>
     <col min="14" max="14" width="19.85546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3237,7 +3274,7 @@
       <c r="Z7" s="1"/>
     </row>
     <row r="8" spans="1:26" ht="15.75" thickBot="1">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="5" t="s">
         <v>0</v>
       </c>
       <c r="B8" s="1"/>
@@ -3273,18 +3310,14 @@
       <c r="B9" s="3"/>
       <c r="C9" s="2"/>
       <c r="D9" s="1"/>
-      <c r="E9" s="46" t="s">
+      <c r="E9" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="F9" s="46"/>
-      <c r="G9" s="46"/>
-      <c r="H9" s="1"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="49"/>
+      <c r="H9" s="43"/>
       <c r="I9" s="1"/>
-      <c r="J9" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="K9" s="3"/>
-      <c r="L9" s="2"/>
+      <c r="J9" s="1"/>
       <c r="M9" s="1"/>
       <c r="N9" s="1"/>
       <c r="O9" s="1"/>
@@ -3301,14 +3334,14 @@
       <c r="Z9" s="1"/>
     </row>
     <row r="10" spans="1:26" ht="15.75" thickBot="1">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="1"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="43" t="s">
         <v>4</v>
-      </c>
-      <c r="B10" s="1"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="45" t="s">
-        <v>5</v>
       </c>
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
@@ -3332,45 +3365,45 @@
       <c r="Y10" s="1"/>
       <c r="Z10" s="1"/>
     </row>
-    <row r="11" spans="1:26" ht="15.75" thickBot="1">
-      <c r="A11" s="21" t="s">
+    <row r="11" spans="1:26" ht="30.75" thickBot="1">
+      <c r="A11" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="C11" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="22" t="s">
+      <c r="D11" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="D11" s="22" t="s">
+      <c r="E11" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="E11" s="21" t="s">
+      <c r="F11" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="F11" s="21" t="s">
+      <c r="G11" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="G11" s="26" t="s">
+      <c r="H11" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="H11" s="24" t="s">
+      <c r="I11" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="I11" s="24" t="s">
+      <c r="J11" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="J11" s="26" t="s">
+      <c r="K11" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="K11" s="22" t="s">
+      <c r="L11" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="L11" s="22" t="s">
+      <c r="M11" s="45" t="s">
         <v>17</v>
-      </c>
-      <c r="M11" s="22" t="s">
-        <v>18</v>
       </c>
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
@@ -3387,23 +3420,22 @@
       <c r="Z11" s="1"/>
     </row>
     <row r="12" spans="1:26" ht="15.75">
-      <c r="A12" s="19">
+      <c r="A12" s="18">
         <v>1</v>
       </c>
-      <c r="B12" s="14"/>
+      <c r="B12" s="13"/>
       <c r="C12" s="13"/>
       <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="J12" s="13"/>
-      <c r="K12" s="38"/>
-      <c r="L12" s="41"/>
-      <c r="M12" s="41"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="12"/>
+      <c r="I12" s="12"/>
+      <c r="J12" s="12"/>
+      <c r="K12" s="36"/>
+      <c r="L12" s="39"/>
+      <c r="M12" s="39"/>
+      <c r="N12" s="44"/>
       <c r="Q12" s="1"/>
       <c r="R12" s="1"/>
       <c r="S12" s="1"/>
@@ -3416,23 +3448,22 @@
       <c r="Z12" s="1"/>
     </row>
     <row r="13" spans="1:26" ht="15.75">
-      <c r="A13" s="18">
+      <c r="A13" s="17">
         <v>2</v>
       </c>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="15"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="15"/>
-      <c r="I13" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="J13" s="15"/>
-      <c r="K13" s="39"/>
-      <c r="L13" s="40"/>
-      <c r="M13" s="42"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14"/>
+      <c r="F13" s="14"/>
+      <c r="G13" s="14"/>
+      <c r="H13" s="14"/>
+      <c r="I13" s="14"/>
+      <c r="J13" s="14"/>
+      <c r="K13" s="38"/>
+      <c r="L13" s="38"/>
+      <c r="M13" s="40"/>
+      <c r="N13" s="44"/>
       <c r="Q13" s="1"/>
       <c r="R13" s="1"/>
       <c r="S13" s="1"/>
@@ -3445,23 +3476,22 @@
       <c r="Z13" s="1"/>
     </row>
     <row r="14" spans="1:26" ht="15.75">
-      <c r="A14" s="17">
+      <c r="A14" s="16">
         <v>3</v>
       </c>
-      <c r="B14" s="14"/>
+      <c r="B14" s="13"/>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="13"/>
-      <c r="H14" s="13"/>
-      <c r="I14" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="J14" s="13"/>
-      <c r="K14" s="38"/>
-      <c r="L14" s="41"/>
-      <c r="M14" s="41"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="12"/>
+      <c r="H14" s="12"/>
+      <c r="I14" s="12"/>
+      <c r="J14" s="12"/>
+      <c r="K14" s="36"/>
+      <c r="L14" s="39"/>
+      <c r="M14" s="39"/>
+      <c r="N14" s="44"/>
       <c r="Q14" s="1"/>
       <c r="R14" s="1"/>
       <c r="S14" s="1"/>
@@ -3474,23 +3504,22 @@
       <c r="Z14" s="1"/>
     </row>
     <row r="15" spans="1:26" ht="15.75">
-      <c r="A15" s="18">
+      <c r="A15" s="17">
         <v>4</v>
       </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
-      <c r="I15" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="J15" s="15"/>
-      <c r="K15" s="39"/>
-      <c r="L15" s="40"/>
-      <c r="M15" s="42"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="14"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="14"/>
+      <c r="H15" s="14"/>
+      <c r="I15" s="14"/>
+      <c r="J15" s="14"/>
+      <c r="K15" s="37"/>
+      <c r="L15" s="38"/>
+      <c r="M15" s="40"/>
+      <c r="N15" s="44"/>
       <c r="Q15" s="1"/>
       <c r="R15" s="1"/>
       <c r="S15" s="1"/>
@@ -3503,23 +3532,22 @@
       <c r="Z15" s="1"/>
     </row>
     <row r="16" spans="1:26" ht="15.75">
-      <c r="A16" s="16">
+      <c r="A16" s="15">
         <v>5</v>
       </c>
-      <c r="B16" s="14"/>
+      <c r="B16" s="13"/>
       <c r="C16" s="13"/>
       <c r="D16" s="13"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="13"/>
-      <c r="H16" s="13"/>
-      <c r="I16" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="J16" s="13"/>
-      <c r="K16" s="38"/>
-      <c r="L16" s="44"/>
-      <c r="M16" s="41"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="12"/>
+      <c r="J16" s="12"/>
+      <c r="K16" s="36"/>
+      <c r="L16" s="39"/>
+      <c r="M16" s="39"/>
+      <c r="N16" s="44"/>
       <c r="Q16" s="1"/>
       <c r="R16" s="1"/>
       <c r="S16" s="1"/>
@@ -3532,23 +3560,22 @@
       <c r="Z16" s="1"/>
     </row>
     <row r="17" spans="1:26" ht="15.75">
-      <c r="A17" s="18">
+      <c r="A17" s="17">
         <v>6</v>
       </c>
-      <c r="B17" s="15"/>
-      <c r="C17" s="15"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="8"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="15"/>
-      <c r="I17" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="J17" s="15"/>
-      <c r="K17" s="39"/>
-      <c r="L17" s="40"/>
-      <c r="M17" s="42"/>
+      <c r="B17" s="14"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="14"/>
+      <c r="E17" s="14"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="14"/>
+      <c r="H17" s="14"/>
+      <c r="I17" s="14"/>
+      <c r="J17" s="14"/>
+      <c r="K17" s="37"/>
+      <c r="L17" s="38"/>
+      <c r="M17" s="40"/>
+      <c r="N17" s="44"/>
       <c r="Q17" s="1"/>
       <c r="R17" s="1"/>
       <c r="S17" s="1"/>
@@ -3561,24 +3588,22 @@
       <c r="Z17" s="1"/>
     </row>
     <row r="18" spans="1:26" ht="15.75">
-      <c r="A18" s="17">
+      <c r="A18" s="16">
         <v>7</v>
       </c>
-      <c r="B18" s="14"/>
+      <c r="B18" s="13"/>
       <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="13"/>
-      <c r="H18" s="13"/>
-      <c r="I18" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="J18" s="13"/>
-      <c r="K18" s="38"/>
-      <c r="L18" s="41"/>
-      <c r="M18" s="41"/>
-      <c r="N18" s="1"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="12"/>
+      <c r="I18" s="12"/>
+      <c r="J18" s="12"/>
+      <c r="K18" s="36"/>
+      <c r="L18" s="39"/>
+      <c r="M18" s="39"/>
+      <c r="N18" s="44"/>
       <c r="O18" s="1"/>
       <c r="P18" s="1"/>
       <c r="Q18" s="1"/>
@@ -3593,23 +3618,21 @@
       <c r="Z18" s="1"/>
     </row>
     <row r="19" spans="1:26" ht="16.5" thickBot="1">
-      <c r="A19" s="18">
+      <c r="A19" s="17">
         <v>8</v>
       </c>
-      <c r="B19" s="15"/>
-      <c r="C19" s="15"/>
-      <c r="D19" s="15"/>
-      <c r="E19" s="15"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="15"/>
-      <c r="H19" s="15"/>
-      <c r="I19" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="J19" s="15"/>
-      <c r="K19" s="39"/>
-      <c r="L19" s="40"/>
-      <c r="M19" s="42"/>
+      <c r="B19" s="14"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="14"/>
+      <c r="H19" s="14"/>
+      <c r="I19" s="14"/>
+      <c r="J19" s="14"/>
+      <c r="K19" s="37"/>
+      <c r="L19" s="38"/>
+      <c r="M19" s="40"/>
       <c r="N19" s="1"/>
       <c r="O19" s="1"/>
       <c r="P19" s="1"/>
@@ -3625,25 +3648,23 @@
       <c r="Z19" s="1"/>
     </row>
     <row r="20" spans="1:26" ht="16.5" thickBot="1">
-      <c r="A20" s="16">
+      <c r="A20" s="15">
         <v>9</v>
       </c>
-      <c r="B20" s="14"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="7"/>
-      <c r="G20" s="13"/>
-      <c r="H20" s="13"/>
-      <c r="I20" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="J20" s="13"/>
-      <c r="K20" s="38"/>
-      <c r="L20" s="44"/>
-      <c r="M20" s="41"/>
-      <c r="N20" s="27" t="s">
-        <v>20</v>
+      <c r="B20" s="13"/>
+      <c r="C20" s="12"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="12"/>
+      <c r="I20" s="12"/>
+      <c r="J20" s="12"/>
+      <c r="K20" s="36"/>
+      <c r="L20" s="42"/>
+      <c r="M20" s="39"/>
+      <c r="N20" s="25" t="s">
+        <v>18</v>
       </c>
       <c r="O20" s="1"/>
       <c r="P20" s="1"/>
@@ -3659,31 +3680,29 @@
       <c r="Z20" s="1"/>
     </row>
     <row r="21" spans="1:26" ht="16.5" thickBot="1">
-      <c r="A21" s="18">
+      <c r="A21" s="17">
         <v>10</v>
       </c>
-      <c r="B21" s="15"/>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="8"/>
-      <c r="G21" s="15"/>
-      <c r="H21" s="15"/>
-      <c r="I21" s="15" t="s">
+      <c r="B21" s="14"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="14"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="14"/>
+      <c r="H21" s="14"/>
+      <c r="I21" s="14"/>
+      <c r="J21" s="14"/>
+      <c r="K21" s="37"/>
+      <c r="L21" s="38"/>
+      <c r="M21" s="40"/>
+      <c r="N21" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="J21" s="15"/>
-      <c r="K21" s="39"/>
-      <c r="L21" s="40"/>
-      <c r="M21" s="42"/>
-      <c r="N21" s="25" t="s">
-        <v>21</v>
-      </c>
-      <c r="O21" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="P21" s="25"/>
-      <c r="Q21" s="25"/>
+      <c r="O21" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="P21" s="24"/>
+      <c r="Q21" s="24"/>
       <c r="R21" s="1"/>
       <c r="S21" s="1"/>
       <c r="T21" s="1"/>
@@ -3695,28 +3714,26 @@
       <c r="Z21" s="1"/>
     </row>
     <row r="22" spans="1:26" ht="15.75">
-      <c r="A22" s="17">
+      <c r="A22" s="16">
         <v>11</v>
       </c>
-      <c r="B22" s="14"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="7"/>
-      <c r="G22" s="13"/>
-      <c r="H22" s="13"/>
-      <c r="I22" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="J22" s="13"/>
-      <c r="K22" s="38"/>
-      <c r="L22" s="41"/>
-      <c r="M22" s="41"/>
-      <c r="N22" s="32" t="s">
-        <v>23</v>
-      </c>
-      <c r="O22" s="28" t="s">
-        <v>24</v>
+      <c r="B22" s="13"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="12"/>
+      <c r="F22" s="6"/>
+      <c r="G22" s="12"/>
+      <c r="H22" s="12"/>
+      <c r="I22" s="12"/>
+      <c r="J22" s="12"/>
+      <c r="K22" s="36"/>
+      <c r="L22" s="39"/>
+      <c r="M22" s="39"/>
+      <c r="N22" s="30" t="s">
+        <v>21</v>
+      </c>
+      <c r="O22" s="26" t="s">
+        <v>22</v>
       </c>
       <c r="P22" s="1"/>
       <c r="Q22" s="1"/>
@@ -3731,28 +3748,26 @@
       <c r="Z22" s="1"/>
     </row>
     <row r="23" spans="1:26" ht="15.75">
-      <c r="A23" s="18">
+      <c r="A23" s="17">
         <v>12</v>
       </c>
-      <c r="B23" s="15"/>
-      <c r="C23" s="15"/>
-      <c r="D23" s="15"/>
-      <c r="E23" s="15"/>
-      <c r="F23" s="8"/>
-      <c r="G23" s="15"/>
-      <c r="H23" s="15"/>
-      <c r="I23" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="J23" s="15"/>
-      <c r="K23" s="39"/>
-      <c r="L23" s="40"/>
-      <c r="M23" s="42"/>
-      <c r="N23" s="33" t="s">
-        <v>25</v>
-      </c>
-      <c r="O23" s="29" t="s">
-        <v>26</v>
+      <c r="B23" s="14"/>
+      <c r="C23" s="14"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="14"/>
+      <c r="F23" s="7"/>
+      <c r="G23" s="14"/>
+      <c r="H23" s="14"/>
+      <c r="I23" s="14"/>
+      <c r="J23" s="14"/>
+      <c r="K23" s="37"/>
+      <c r="L23" s="38"/>
+      <c r="M23" s="40"/>
+      <c r="N23" s="31" t="s">
+        <v>23</v>
+      </c>
+      <c r="O23" s="27" t="s">
+        <v>24</v>
       </c>
       <c r="P23" s="1"/>
       <c r="Q23" s="1"/>
@@ -3767,28 +3782,26 @@
       <c r="Z23" s="1"/>
     </row>
     <row r="24" spans="1:26" ht="16.5" thickBot="1">
-      <c r="A24" s="16">
+      <c r="A24" s="15">
         <v>13</v>
       </c>
-      <c r="B24" s="14"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="7"/>
-      <c r="G24" s="13"/>
-      <c r="H24" s="13"/>
-      <c r="I24" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="J24" s="13"/>
-      <c r="K24" s="38"/>
-      <c r="L24" s="44"/>
-      <c r="M24" s="41"/>
-      <c r="N24" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="O24" s="29" t="s">
-        <v>28</v>
+      <c r="B24" s="13"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="12"/>
+      <c r="H24" s="12"/>
+      <c r="I24" s="12"/>
+      <c r="J24" s="12"/>
+      <c r="K24" s="36"/>
+      <c r="L24" s="42"/>
+      <c r="M24" s="39"/>
+      <c r="N24" s="32" t="s">
+        <v>25</v>
+      </c>
+      <c r="O24" s="27" t="s">
+        <v>26</v>
       </c>
       <c r="P24" s="1"/>
       <c r="Q24" s="1"/>
@@ -3803,25 +3816,23 @@
       <c r="Z24" s="1"/>
     </row>
     <row r="25" spans="1:26" ht="16.5" thickBot="1">
-      <c r="A25" s="18">
+      <c r="A25" s="17">
         <v>14</v>
       </c>
-      <c r="B25" s="15"/>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
-      <c r="E25" s="15"/>
-      <c r="F25" s="8"/>
-      <c r="G25" s="15"/>
-      <c r="H25" s="15"/>
-      <c r="I25" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="J25" s="15"/>
-      <c r="K25" s="39"/>
-      <c r="L25" s="40"/>
-      <c r="M25" s="42"/>
-      <c r="N25" s="35"/>
-      <c r="O25" s="29"/>
+      <c r="B25" s="14"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="14"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="14"/>
+      <c r="H25" s="14"/>
+      <c r="I25" s="14"/>
+      <c r="J25" s="14"/>
+      <c r="K25" s="37"/>
+      <c r="L25" s="38"/>
+      <c r="M25" s="40"/>
+      <c r="N25" s="33"/>
+      <c r="O25" s="27"/>
       <c r="P25" s="1"/>
       <c r="Q25" s="1"/>
       <c r="R25" s="1"/>
@@ -3835,31 +3846,29 @@
       <c r="Z25" s="1"/>
     </row>
     <row r="26" spans="1:26" ht="16.5" thickBot="1">
-      <c r="A26" s="17">
+      <c r="A26" s="16">
         <v>15</v>
       </c>
-      <c r="B26" s="14"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="7"/>
-      <c r="G26" s="13"/>
-      <c r="H26" s="13"/>
-      <c r="I26" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="J26" s="13"/>
-      <c r="K26" s="38"/>
-      <c r="L26" s="41"/>
-      <c r="M26" s="41"/>
-      <c r="N26" s="25" t="s">
-        <v>12</v>
-      </c>
-      <c r="O26" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="P26" s="25"/>
-      <c r="Q26" s="25"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="12"/>
+      <c r="H26" s="12"/>
+      <c r="I26" s="12"/>
+      <c r="J26" s="12"/>
+      <c r="K26" s="36"/>
+      <c r="L26" s="39"/>
+      <c r="M26" s="39"/>
+      <c r="N26" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="O26" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="P26" s="24"/>
+      <c r="Q26" s="24"/>
       <c r="R26" s="1"/>
       <c r="S26" s="1"/>
       <c r="T26" s="1"/>
@@ -3871,25 +3880,23 @@
       <c r="Z26" s="1"/>
     </row>
     <row r="27" spans="1:26" ht="16.5" thickBot="1">
-      <c r="A27" s="18">
+      <c r="A27" s="17">
         <v>16</v>
       </c>
-      <c r="B27" s="15"/>
-      <c r="C27" s="15"/>
-      <c r="D27" s="15"/>
-      <c r="E27" s="15"/>
-      <c r="F27" s="8"/>
-      <c r="G27" s="15"/>
-      <c r="H27" s="15"/>
-      <c r="I27" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="J27" s="15"/>
-      <c r="K27" s="39"/>
-      <c r="L27" s="40"/>
-      <c r="M27" s="42"/>
-      <c r="N27" s="32" t="s">
-        <v>29</v>
+      <c r="B27" s="14"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="14"/>
+      <c r="F27" s="7"/>
+      <c r="G27" s="14"/>
+      <c r="H27" s="14"/>
+      <c r="I27" s="14"/>
+      <c r="J27" s="14"/>
+      <c r="K27" s="37"/>
+      <c r="L27" s="38"/>
+      <c r="M27" s="40"/>
+      <c r="N27" s="30" t="s">
+        <v>28</v>
       </c>
       <c r="O27" s="1"/>
       <c r="P27" s="1"/>
@@ -3905,25 +3912,23 @@
       <c r="Z27" s="1"/>
     </row>
     <row r="28" spans="1:26" ht="15.75">
-      <c r="A28" s="16">
+      <c r="A28" s="15">
         <v>17</v>
       </c>
-      <c r="B28" s="14"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="13"/>
-      <c r="F28" s="7"/>
-      <c r="G28" s="13"/>
-      <c r="H28" s="13"/>
-      <c r="I28" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="J28" s="13"/>
-      <c r="K28" s="38"/>
-      <c r="L28" s="44"/>
-      <c r="M28" s="41"/>
-      <c r="N28" s="32" t="s">
-        <v>30</v>
+      <c r="B28" s="13"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="12"/>
+      <c r="F28" s="6"/>
+      <c r="G28" s="12"/>
+      <c r="H28" s="12"/>
+      <c r="I28" s="12"/>
+      <c r="J28" s="12"/>
+      <c r="K28" s="36"/>
+      <c r="L28" s="42"/>
+      <c r="M28" s="39"/>
+      <c r="N28" s="30" t="s">
+        <v>29</v>
       </c>
       <c r="O28" s="1"/>
       <c r="P28" s="1"/>
@@ -3939,26 +3944,26 @@
       <c r="Z28" s="1"/>
     </row>
     <row r="29" spans="1:26" ht="16.5" thickBot="1">
-      <c r="A29" s="18">
+      <c r="A29" s="17">
         <v>18</v>
       </c>
-      <c r="B29" s="15"/>
-      <c r="C29" s="15"/>
-      <c r="D29" s="15"/>
-      <c r="E29" s="15"/>
-      <c r="F29" s="8"/>
-      <c r="G29" s="8"/>
-      <c r="H29" s="15"/>
-      <c r="I29" s="15"/>
-      <c r="J29" s="15"/>
-      <c r="K29" s="39"/>
-      <c r="L29" s="9"/>
-      <c r="M29" s="9"/>
-      <c r="N29" s="34" t="s">
+      <c r="B29" s="14"/>
+      <c r="C29" s="14"/>
+      <c r="D29" s="14"/>
+      <c r="E29" s="14"/>
+      <c r="F29" s="7"/>
+      <c r="G29" s="7"/>
+      <c r="H29" s="14"/>
+      <c r="I29" s="14"/>
+      <c r="J29" s="14"/>
+      <c r="K29" s="37"/>
+      <c r="L29" s="8"/>
+      <c r="M29" s="8"/>
+      <c r="N29" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="O29" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="O29" s="1" t="s">
-        <v>32</v>
       </c>
       <c r="P29" s="1"/>
       <c r="Q29" s="1"/>
@@ -3973,23 +3978,23 @@
       <c r="Z29" s="1"/>
     </row>
     <row r="30" spans="1:26" ht="16.5" thickBot="1">
-      <c r="A30" s="17">
+      <c r="A30" s="16">
         <v>19</v>
       </c>
-      <c r="B30" s="14"/>
-      <c r="C30" s="13"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
-      <c r="F30" s="7"/>
-      <c r="G30" s="7"/>
-      <c r="H30" s="13"/>
-      <c r="I30" s="14"/>
-      <c r="J30" s="13"/>
-      <c r="K30" s="38"/>
-      <c r="L30" s="12"/>
-      <c r="M30" s="12"/>
-      <c r="N30" s="34" t="s">
-        <v>33</v>
+      <c r="B30" s="13"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="6"/>
+      <c r="G30" s="6"/>
+      <c r="H30" s="12"/>
+      <c r="I30" s="13"/>
+      <c r="J30" s="12"/>
+      <c r="K30" s="36"/>
+      <c r="L30" s="11"/>
+      <c r="M30" s="11"/>
+      <c r="N30" s="32" t="s">
+        <v>32</v>
       </c>
       <c r="O30" s="1"/>
       <c r="P30" s="1"/>
@@ -4005,23 +4010,23 @@
       <c r="Z30" s="1"/>
     </row>
     <row r="31" spans="1:26" ht="16.5" thickBot="1">
-      <c r="A31" s="18">
+      <c r="A31" s="17">
         <v>20</v>
       </c>
-      <c r="B31" s="15"/>
-      <c r="C31" s="15"/>
-      <c r="D31" s="15"/>
-      <c r="E31" s="15"/>
-      <c r="F31" s="8"/>
-      <c r="G31" s="8"/>
-      <c r="H31" s="15"/>
-      <c r="I31" s="15"/>
-      <c r="J31" s="15"/>
-      <c r="K31" s="39"/>
-      <c r="L31" s="9"/>
-      <c r="M31" s="9"/>
-      <c r="N31" s="34" t="s">
-        <v>34</v>
+      <c r="B31" s="14"/>
+      <c r="C31" s="14"/>
+      <c r="D31" s="14"/>
+      <c r="E31" s="14"/>
+      <c r="F31" s="7"/>
+      <c r="G31" s="7"/>
+      <c r="H31" s="14"/>
+      <c r="I31" s="14"/>
+      <c r="J31" s="14"/>
+      <c r="K31" s="37"/>
+      <c r="L31" s="8"/>
+      <c r="M31" s="8"/>
+      <c r="N31" s="32" t="s">
+        <v>33</v>
       </c>
       <c r="O31" s="1"/>
       <c r="P31" s="1"/>
@@ -4037,23 +4042,23 @@
       <c r="Z31" s="1"/>
     </row>
     <row r="32" spans="1:26" ht="16.5" thickBot="1">
-      <c r="A32" s="16">
+      <c r="A32" s="15">
         <v>21</v>
       </c>
-      <c r="B32" s="14"/>
-      <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="7"/>
-      <c r="G32" s="7"/>
-      <c r="H32" s="13"/>
-      <c r="I32" s="14"/>
-      <c r="J32" s="13"/>
-      <c r="K32" s="38"/>
-      <c r="L32" s="11"/>
-      <c r="M32" s="12"/>
-      <c r="N32" s="34" t="s">
-        <v>35</v>
+      <c r="B32" s="13"/>
+      <c r="C32" s="12"/>
+      <c r="D32" s="12"/>
+      <c r="E32" s="12"/>
+      <c r="F32" s="6"/>
+      <c r="G32" s="6"/>
+      <c r="H32" s="12"/>
+      <c r="I32" s="13"/>
+      <c r="J32" s="12"/>
+      <c r="K32" s="36"/>
+      <c r="L32" s="10"/>
+      <c r="M32" s="11"/>
+      <c r="N32" s="32" t="s">
+        <v>34</v>
       </c>
       <c r="O32" s="1"/>
       <c r="P32" s="1"/>
@@ -4069,23 +4074,23 @@
       <c r="Z32" s="1"/>
     </row>
     <row r="33" spans="1:26" ht="16.5" thickBot="1">
-      <c r="A33" s="18">
+      <c r="A33" s="17">
         <v>22</v>
       </c>
-      <c r="B33" s="15"/>
-      <c r="C33" s="15"/>
-      <c r="D33" s="15"/>
-      <c r="E33" s="15"/>
-      <c r="F33" s="8"/>
-      <c r="G33" s="8"/>
-      <c r="H33" s="15"/>
-      <c r="I33" s="15"/>
-      <c r="J33" s="15"/>
-      <c r="K33" s="39"/>
-      <c r="L33" s="9"/>
-      <c r="M33" s="43"/>
-      <c r="N33" s="34" t="s">
-        <v>36</v>
+      <c r="B33" s="14"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="14"/>
+      <c r="F33" s="7"/>
+      <c r="G33" s="7"/>
+      <c r="H33" s="14"/>
+      <c r="I33" s="14"/>
+      <c r="J33" s="14"/>
+      <c r="K33" s="37"/>
+      <c r="L33" s="8"/>
+      <c r="M33" s="41"/>
+      <c r="N33" s="32" t="s">
+        <v>35</v>
       </c>
       <c r="O33" s="1"/>
       <c r="P33" s="1"/>
@@ -4101,21 +4106,21 @@
       <c r="Z33" s="1"/>
     </row>
     <row r="34" spans="1:26" ht="15.75">
-      <c r="A34" s="17">
+      <c r="A34" s="16">
         <v>23</v>
       </c>
-      <c r="B34" s="14"/>
-      <c r="C34" s="13"/>
-      <c r="D34" s="13"/>
-      <c r="E34" s="13"/>
-      <c r="F34" s="7"/>
-      <c r="G34" s="7"/>
-      <c r="H34" s="13"/>
-      <c r="I34" s="14"/>
-      <c r="J34" s="13"/>
-      <c r="K34" s="38"/>
-      <c r="L34" s="12"/>
-      <c r="M34" s="12"/>
+      <c r="B34" s="13"/>
+      <c r="C34" s="12"/>
+      <c r="D34" s="12"/>
+      <c r="E34" s="12"/>
+      <c r="F34" s="6"/>
+      <c r="G34" s="6"/>
+      <c r="H34" s="12"/>
+      <c r="I34" s="13"/>
+      <c r="J34" s="12"/>
+      <c r="K34" s="36"/>
+      <c r="L34" s="11"/>
+      <c r="M34" s="11"/>
       <c r="N34" s="1"/>
       <c r="O34" s="1"/>
       <c r="P34" s="1"/>
@@ -4131,21 +4136,21 @@
       <c r="Z34" s="1"/>
     </row>
     <row r="35" spans="1:26" ht="15.75">
-      <c r="A35" s="18">
+      <c r="A35" s="17">
         <v>24</v>
       </c>
-      <c r="B35" s="15"/>
-      <c r="C35" s="15"/>
-      <c r="D35" s="15"/>
-      <c r="E35" s="15"/>
-      <c r="F35" s="8"/>
-      <c r="G35" s="8"/>
-      <c r="H35" s="15"/>
-      <c r="I35" s="15"/>
-      <c r="J35" s="15"/>
-      <c r="K35" s="39"/>
-      <c r="L35" s="9"/>
-      <c r="M35" s="9"/>
+      <c r="B35" s="14"/>
+      <c r="C35" s="14"/>
+      <c r="D35" s="14"/>
+      <c r="E35" s="14"/>
+      <c r="F35" s="7"/>
+      <c r="G35" s="7"/>
+      <c r="H35" s="14"/>
+      <c r="I35" s="14"/>
+      <c r="J35" s="14"/>
+      <c r="K35" s="37"/>
+      <c r="L35" s="8"/>
+      <c r="M35" s="8"/>
       <c r="N35" s="1"/>
       <c r="O35" s="1"/>
       <c r="P35" s="1"/>
@@ -4161,21 +4166,21 @@
       <c r="Z35" s="1"/>
     </row>
     <row r="36" spans="1:26" ht="15.75">
-      <c r="A36" s="16">
+      <c r="A36" s="15">
         <v>25</v>
       </c>
-      <c r="B36" s="14"/>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
-      <c r="E36" s="13"/>
-      <c r="F36" s="7"/>
-      <c r="G36" s="7"/>
-      <c r="H36" s="13"/>
-      <c r="I36" s="14"/>
-      <c r="J36" s="13"/>
-      <c r="K36" s="38"/>
-      <c r="L36" s="11"/>
-      <c r="M36" s="12"/>
+      <c r="B36" s="13"/>
+      <c r="C36" s="12"/>
+      <c r="D36" s="12"/>
+      <c r="E36" s="12"/>
+      <c r="F36" s="6"/>
+      <c r="G36" s="6"/>
+      <c r="H36" s="12"/>
+      <c r="I36" s="13"/>
+      <c r="J36" s="12"/>
+      <c r="K36" s="36"/>
+      <c r="L36" s="10"/>
+      <c r="M36" s="11"/>
       <c r="N36" s="1"/>
       <c r="O36" s="1"/>
       <c r="P36" s="1"/>
@@ -4191,21 +4196,21 @@
       <c r="Z36" s="1"/>
     </row>
     <row r="37" spans="1:26" ht="15.75">
-      <c r="A37" s="18">
+      <c r="A37" s="17">
         <v>26</v>
       </c>
-      <c r="B37" s="15"/>
-      <c r="C37" s="15"/>
-      <c r="D37" s="15"/>
-      <c r="E37" s="15"/>
-      <c r="F37" s="8"/>
-      <c r="G37" s="8"/>
-      <c r="H37" s="15"/>
-      <c r="I37" s="15"/>
-      <c r="J37" s="15"/>
-      <c r="K37" s="39"/>
-      <c r="L37" s="9"/>
-      <c r="M37" s="9"/>
+      <c r="B37" s="14"/>
+      <c r="C37" s="14"/>
+      <c r="D37" s="14"/>
+      <c r="E37" s="14"/>
+      <c r="F37" s="7"/>
+      <c r="G37" s="7"/>
+      <c r="H37" s="14"/>
+      <c r="I37" s="14"/>
+      <c r="J37" s="14"/>
+      <c r="K37" s="37"/>
+      <c r="L37" s="8"/>
+      <c r="M37" s="8"/>
       <c r="N37" s="1"/>
       <c r="O37" s="1"/>
       <c r="P37" s="1"/>
@@ -4221,21 +4226,21 @@
       <c r="Z37" s="1"/>
     </row>
     <row r="38" spans="1:26" ht="15.75">
-      <c r="A38" s="17">
+      <c r="A38" s="16">
         <v>27</v>
       </c>
-      <c r="B38" s="14"/>
-      <c r="C38" s="13"/>
-      <c r="D38" s="13"/>
-      <c r="E38" s="13"/>
-      <c r="F38" s="7"/>
-      <c r="G38" s="7"/>
-      <c r="H38" s="13"/>
-      <c r="I38" s="14"/>
-      <c r="J38" s="13"/>
-      <c r="K38" s="38"/>
-      <c r="L38" s="12"/>
-      <c r="M38" s="12"/>
+      <c r="B38" s="13"/>
+      <c r="C38" s="12"/>
+      <c r="D38" s="12"/>
+      <c r="E38" s="12"/>
+      <c r="F38" s="6"/>
+      <c r="G38" s="6"/>
+      <c r="H38" s="12"/>
+      <c r="I38" s="13"/>
+      <c r="J38" s="12"/>
+      <c r="K38" s="36"/>
+      <c r="L38" s="11"/>
+      <c r="M38" s="11"/>
       <c r="N38" s="1"/>
       <c r="O38" s="1"/>
       <c r="P38" s="1"/>
@@ -4251,21 +4256,21 @@
       <c r="Z38" s="1"/>
     </row>
     <row r="39" spans="1:26" ht="15.75">
-      <c r="A39" s="18">
+      <c r="A39" s="17">
         <v>28</v>
       </c>
-      <c r="B39" s="15"/>
-      <c r="C39" s="15"/>
-      <c r="D39" s="15"/>
-      <c r="E39" s="15"/>
-      <c r="F39" s="8"/>
-      <c r="G39" s="8"/>
-      <c r="H39" s="15"/>
-      <c r="I39" s="15"/>
-      <c r="J39" s="15"/>
-      <c r="K39" s="39"/>
-      <c r="L39" s="9"/>
-      <c r="M39" s="9"/>
+      <c r="B39" s="14"/>
+      <c r="C39" s="14"/>
+      <c r="D39" s="14"/>
+      <c r="E39" s="14"/>
+      <c r="F39" s="7"/>
+      <c r="G39" s="7"/>
+      <c r="H39" s="14"/>
+      <c r="I39" s="14"/>
+      <c r="J39" s="14"/>
+      <c r="K39" s="37"/>
+      <c r="L39" s="8"/>
+      <c r="M39" s="8"/>
       <c r="N39" s="1"/>
       <c r="O39" s="1"/>
       <c r="P39" s="1"/>
@@ -4281,21 +4286,21 @@
       <c r="Z39" s="1"/>
     </row>
     <row r="40" spans="1:26" ht="15.75">
-      <c r="A40" s="16">
+      <c r="A40" s="15">
         <v>29</v>
       </c>
-      <c r="B40" s="14"/>
-      <c r="C40" s="13"/>
-      <c r="D40" s="13"/>
-      <c r="E40" s="13"/>
-      <c r="F40" s="7"/>
-      <c r="G40" s="7"/>
-      <c r="H40" s="13"/>
-      <c r="I40" s="14"/>
-      <c r="J40" s="13"/>
-      <c r="K40" s="38"/>
-      <c r="L40" s="11"/>
-      <c r="M40" s="12"/>
+      <c r="B40" s="13"/>
+      <c r="C40" s="12"/>
+      <c r="D40" s="12"/>
+      <c r="E40" s="12"/>
+      <c r="F40" s="6"/>
+      <c r="G40" s="6"/>
+      <c r="H40" s="12"/>
+      <c r="I40" s="13"/>
+      <c r="J40" s="12"/>
+      <c r="K40" s="36"/>
+      <c r="L40" s="10"/>
+      <c r="M40" s="11"/>
       <c r="N40" s="1"/>
       <c r="O40" s="1"/>
       <c r="P40" s="1"/>
@@ -4311,21 +4316,21 @@
       <c r="Z40" s="1"/>
     </row>
     <row r="41" spans="1:26" ht="15.75">
-      <c r="A41" s="18">
+      <c r="A41" s="17">
         <v>30</v>
       </c>
-      <c r="B41" s="15"/>
-      <c r="C41" s="15"/>
-      <c r="D41" s="15"/>
-      <c r="E41" s="15"/>
-      <c r="F41" s="8"/>
-      <c r="G41" s="8"/>
-      <c r="H41" s="15"/>
-      <c r="I41" s="15"/>
-      <c r="J41" s="15"/>
-      <c r="K41" s="39"/>
-      <c r="L41" s="9"/>
-      <c r="M41" s="9"/>
+      <c r="B41" s="14"/>
+      <c r="C41" s="14"/>
+      <c r="D41" s="14"/>
+      <c r="E41" s="14"/>
+      <c r="F41" s="7"/>
+      <c r="G41" s="7"/>
+      <c r="H41" s="14"/>
+      <c r="I41" s="14"/>
+      <c r="J41" s="14"/>
+      <c r="K41" s="37"/>
+      <c r="L41" s="8"/>
+      <c r="M41" s="8"/>
       <c r="N41" s="1"/>
       <c r="O41" s="1"/>
       <c r="P41" s="1"/>
@@ -4341,21 +4346,21 @@
       <c r="Z41" s="1"/>
     </row>
     <row r="42" spans="1:26" ht="15.75">
-      <c r="A42" s="17">
+      <c r="A42" s="16">
         <v>31</v>
       </c>
-      <c r="B42" s="14"/>
-      <c r="C42" s="13"/>
-      <c r="D42" s="13"/>
-      <c r="E42" s="13"/>
-      <c r="F42" s="7"/>
-      <c r="G42" s="7"/>
-      <c r="H42" s="13"/>
-      <c r="I42" s="14"/>
-      <c r="J42" s="13"/>
-      <c r="K42" s="38"/>
-      <c r="L42" s="12"/>
-      <c r="M42" s="12"/>
+      <c r="B42" s="13"/>
+      <c r="C42" s="12"/>
+      <c r="D42" s="12"/>
+      <c r="E42" s="12"/>
+      <c r="F42" s="6"/>
+      <c r="G42" s="6"/>
+      <c r="H42" s="12"/>
+      <c r="I42" s="13"/>
+      <c r="J42" s="12"/>
+      <c r="K42" s="36"/>
+      <c r="L42" s="11"/>
+      <c r="M42" s="11"/>
       <c r="N42" s="1"/>
       <c r="O42" s="1"/>
       <c r="P42" s="1"/>
@@ -4371,21 +4376,21 @@
       <c r="Z42" s="1"/>
     </row>
     <row r="43" spans="1:26" ht="15.75">
-      <c r="A43" s="18">
+      <c r="A43" s="17">
         <v>32</v>
       </c>
-      <c r="B43" s="15"/>
-      <c r="C43" s="15"/>
-      <c r="D43" s="15"/>
-      <c r="E43" s="15"/>
-      <c r="F43" s="8"/>
-      <c r="G43" s="8"/>
-      <c r="H43" s="15"/>
-      <c r="I43" s="15"/>
-      <c r="J43" s="15"/>
-      <c r="K43" s="39"/>
-      <c r="L43" s="9"/>
-      <c r="M43" s="9"/>
+      <c r="B43" s="14"/>
+      <c r="C43" s="14"/>
+      <c r="D43" s="14"/>
+      <c r="E43" s="14"/>
+      <c r="F43" s="7"/>
+      <c r="G43" s="7"/>
+      <c r="H43" s="14"/>
+      <c r="I43" s="14"/>
+      <c r="J43" s="14"/>
+      <c r="K43" s="37"/>
+      <c r="L43" s="8"/>
+      <c r="M43" s="8"/>
       <c r="N43" s="1"/>
       <c r="O43" s="1"/>
       <c r="P43" s="1"/>
@@ -4401,21 +4406,21 @@
       <c r="Z43" s="1"/>
     </row>
     <row r="44" spans="1:26" ht="15.75">
-      <c r="A44" s="16">
+      <c r="A44" s="15">
         <v>33</v>
       </c>
-      <c r="B44" s="14"/>
-      <c r="C44" s="13"/>
-      <c r="D44" s="13"/>
-      <c r="E44" s="13"/>
-      <c r="F44" s="7"/>
-      <c r="G44" s="7"/>
-      <c r="H44" s="13"/>
-      <c r="I44" s="14"/>
-      <c r="J44" s="13"/>
-      <c r="K44" s="38"/>
-      <c r="L44" s="11"/>
-      <c r="M44" s="12"/>
+      <c r="B44" s="13"/>
+      <c r="C44" s="12"/>
+      <c r="D44" s="12"/>
+      <c r="E44" s="12"/>
+      <c r="F44" s="6"/>
+      <c r="G44" s="6"/>
+      <c r="H44" s="12"/>
+      <c r="I44" s="13"/>
+      <c r="J44" s="12"/>
+      <c r="K44" s="36"/>
+      <c r="L44" s="10"/>
+      <c r="M44" s="11"/>
       <c r="N44" s="1"/>
       <c r="O44" s="1"/>
       <c r="P44" s="1"/>
@@ -4431,21 +4436,21 @@
       <c r="Z44" s="1"/>
     </row>
     <row r="45" spans="1:26" ht="15.75">
-      <c r="A45" s="18">
+      <c r="A45" s="17">
         <v>34</v>
       </c>
-      <c r="B45" s="15"/>
-      <c r="C45" s="15"/>
-      <c r="D45" s="15"/>
-      <c r="E45" s="15"/>
-      <c r="F45" s="8"/>
-      <c r="G45" s="8"/>
-      <c r="H45" s="15"/>
-      <c r="I45" s="15"/>
-      <c r="J45" s="15"/>
-      <c r="K45" s="39"/>
-      <c r="L45" s="9"/>
-      <c r="M45" s="9"/>
+      <c r="B45" s="14"/>
+      <c r="C45" s="14"/>
+      <c r="D45" s="14"/>
+      <c r="E45" s="14"/>
+      <c r="F45" s="7"/>
+      <c r="G45" s="7"/>
+      <c r="H45" s="14"/>
+      <c r="I45" s="14"/>
+      <c r="J45" s="14"/>
+      <c r="K45" s="37"/>
+      <c r="L45" s="8"/>
+      <c r="M45" s="8"/>
       <c r="N45" s="1"/>
       <c r="O45" s="1"/>
       <c r="P45" s="1"/>
@@ -4461,21 +4466,21 @@
       <c r="Z45" s="1"/>
     </row>
     <row r="46" spans="1:26" ht="15.75">
-      <c r="A46" s="17">
+      <c r="A46" s="16">
         <v>35</v>
       </c>
-      <c r="B46" s="14"/>
-      <c r="C46" s="13"/>
-      <c r="D46" s="13"/>
-      <c r="E46" s="13"/>
-      <c r="F46" s="7"/>
-      <c r="G46" s="7"/>
-      <c r="H46" s="13"/>
-      <c r="I46" s="14"/>
-      <c r="J46" s="13"/>
-      <c r="K46" s="38"/>
-      <c r="L46" s="12"/>
-      <c r="M46" s="12"/>
+      <c r="B46" s="13"/>
+      <c r="C46" s="12"/>
+      <c r="D46" s="12"/>
+      <c r="E46" s="12"/>
+      <c r="F46" s="6"/>
+      <c r="G46" s="6"/>
+      <c r="H46" s="12"/>
+      <c r="I46" s="13"/>
+      <c r="J46" s="12"/>
+      <c r="K46" s="36"/>
+      <c r="L46" s="11"/>
+      <c r="M46" s="11"/>
       <c r="N46" s="1"/>
       <c r="O46" s="1"/>
       <c r="P46" s="1"/>
@@ -4491,21 +4496,21 @@
       <c r="Z46" s="1"/>
     </row>
     <row r="47" spans="1:26" ht="15.75">
-      <c r="A47" s="18">
+      <c r="A47" s="17">
         <v>36</v>
       </c>
-      <c r="B47" s="15"/>
-      <c r="C47" s="15"/>
-      <c r="D47" s="15"/>
-      <c r="E47" s="15"/>
-      <c r="F47" s="8"/>
-      <c r="G47" s="8"/>
-      <c r="H47" s="15"/>
-      <c r="I47" s="15"/>
-      <c r="J47" s="15"/>
-      <c r="K47" s="39"/>
-      <c r="L47" s="9"/>
-      <c r="M47" s="9"/>
+      <c r="B47" s="14"/>
+      <c r="C47" s="14"/>
+      <c r="D47" s="14"/>
+      <c r="E47" s="14"/>
+      <c r="F47" s="7"/>
+      <c r="G47" s="7"/>
+      <c r="H47" s="14"/>
+      <c r="I47" s="14"/>
+      <c r="J47" s="14"/>
+      <c r="K47" s="37"/>
+      <c r="L47" s="8"/>
+      <c r="M47" s="8"/>
       <c r="N47" s="1"/>
       <c r="O47" s="1"/>
       <c r="P47" s="1"/>
@@ -4521,21 +4526,21 @@
       <c r="Z47" s="1"/>
     </row>
     <row r="48" spans="1:26" ht="15.75">
-      <c r="A48" s="16">
+      <c r="A48" s="15">
         <v>37</v>
       </c>
-      <c r="B48" s="14"/>
-      <c r="C48" s="13"/>
-      <c r="D48" s="13"/>
-      <c r="E48" s="7"/>
-      <c r="F48" s="7"/>
-      <c r="G48" s="7"/>
-      <c r="H48" s="13"/>
-      <c r="I48" s="13"/>
-      <c r="J48" s="13"/>
-      <c r="K48" s="38"/>
-      <c r="L48" s="11"/>
-      <c r="M48" s="12"/>
+      <c r="B48" s="13"/>
+      <c r="C48" s="12"/>
+      <c r="D48" s="12"/>
+      <c r="E48" s="6"/>
+      <c r="F48" s="6"/>
+      <c r="G48" s="6"/>
+      <c r="H48" s="12"/>
+      <c r="I48" s="12"/>
+      <c r="J48" s="12"/>
+      <c r="K48" s="36"/>
+      <c r="L48" s="10"/>
+      <c r="M48" s="11"/>
       <c r="N48" s="1"/>
       <c r="O48" s="1"/>
       <c r="P48" s="1"/>
@@ -4551,21 +4556,21 @@
       <c r="Z48" s="1"/>
     </row>
     <row r="49" spans="1:26" ht="15.75">
-      <c r="A49" s="18">
+      <c r="A49" s="17">
         <v>38</v>
       </c>
-      <c r="B49" s="15"/>
-      <c r="C49" s="15"/>
-      <c r="D49" s="15"/>
-      <c r="E49" s="8"/>
-      <c r="F49" s="8"/>
-      <c r="G49" s="8"/>
-      <c r="H49" s="15"/>
-      <c r="I49" s="15"/>
-      <c r="J49" s="15"/>
-      <c r="K49" s="39"/>
-      <c r="L49" s="9"/>
-      <c r="M49" s="9"/>
+      <c r="B49" s="14"/>
+      <c r="C49" s="14"/>
+      <c r="D49" s="14"/>
+      <c r="E49" s="7"/>
+      <c r="F49" s="7"/>
+      <c r="G49" s="7"/>
+      <c r="H49" s="14"/>
+      <c r="I49" s="14"/>
+      <c r="J49" s="14"/>
+      <c r="K49" s="37"/>
+      <c r="L49" s="8"/>
+      <c r="M49" s="8"/>
       <c r="N49" s="1"/>
       <c r="O49" s="1"/>
       <c r="P49" s="1"/>
@@ -4581,21 +4586,21 @@
       <c r="Z49" s="1"/>
     </row>
     <row r="50" spans="1:26" ht="15.75">
-      <c r="A50" s="17">
+      <c r="A50" s="16">
         <v>39</v>
       </c>
-      <c r="B50" s="14"/>
-      <c r="C50" s="13"/>
-      <c r="D50" s="13"/>
-      <c r="E50" s="7"/>
-      <c r="F50" s="7"/>
-      <c r="G50" s="7"/>
-      <c r="H50" s="13"/>
-      <c r="I50" s="13"/>
-      <c r="J50" s="13"/>
-      <c r="K50" s="38"/>
-      <c r="L50" s="12"/>
-      <c r="M50" s="12"/>
+      <c r="B50" s="13"/>
+      <c r="C50" s="12"/>
+      <c r="D50" s="12"/>
+      <c r="E50" s="6"/>
+      <c r="F50" s="6"/>
+      <c r="G50" s="6"/>
+      <c r="H50" s="12"/>
+      <c r="I50" s="12"/>
+      <c r="J50" s="12"/>
+      <c r="K50" s="36"/>
+      <c r="L50" s="11"/>
+      <c r="M50" s="11"/>
       <c r="N50" s="1"/>
       <c r="O50" s="1"/>
       <c r="P50" s="1"/>
@@ -4611,21 +4616,21 @@
       <c r="Z50" s="1"/>
     </row>
     <row r="51" spans="1:26" ht="15.75">
-      <c r="A51" s="18">
+      <c r="A51" s="17">
         <v>40</v>
       </c>
-      <c r="B51" s="15"/>
-      <c r="C51" s="15"/>
-      <c r="D51" s="15"/>
-      <c r="E51" s="8"/>
-      <c r="F51" s="8"/>
-      <c r="G51" s="8"/>
-      <c r="H51" s="15"/>
-      <c r="I51" s="15"/>
-      <c r="J51" s="15"/>
-      <c r="K51" s="39"/>
-      <c r="L51" s="9"/>
-      <c r="M51" s="9"/>
+      <c r="B51" s="14"/>
+      <c r="C51" s="14"/>
+      <c r="D51" s="14"/>
+      <c r="E51" s="7"/>
+      <c r="F51" s="7"/>
+      <c r="G51" s="7"/>
+      <c r="H51" s="14"/>
+      <c r="I51" s="14"/>
+      <c r="J51" s="14"/>
+      <c r="K51" s="37"/>
+      <c r="L51" s="8"/>
+      <c r="M51" s="8"/>
       <c r="N51" s="1"/>
       <c r="O51" s="1"/>
       <c r="P51" s="1"/>
@@ -4641,21 +4646,21 @@
       <c r="Z51" s="1"/>
     </row>
     <row r="52" spans="1:26" ht="15.75">
-      <c r="A52" s="16">
+      <c r="A52" s="15">
         <v>41</v>
       </c>
-      <c r="B52" s="14"/>
-      <c r="C52" s="13"/>
-      <c r="D52" s="13"/>
-      <c r="E52" s="7"/>
-      <c r="F52" s="7"/>
-      <c r="G52" s="7"/>
-      <c r="H52" s="13"/>
-      <c r="I52" s="13"/>
-      <c r="J52" s="13"/>
-      <c r="K52" s="38"/>
-      <c r="L52" s="11"/>
-      <c r="M52" s="12"/>
+      <c r="B52" s="13"/>
+      <c r="C52" s="12"/>
+      <c r="D52" s="12"/>
+      <c r="E52" s="6"/>
+      <c r="F52" s="6"/>
+      <c r="G52" s="6"/>
+      <c r="H52" s="12"/>
+      <c r="I52" s="12"/>
+      <c r="J52" s="12"/>
+      <c r="K52" s="36"/>
+      <c r="L52" s="10"/>
+      <c r="M52" s="11"/>
       <c r="N52" s="1"/>
       <c r="O52" s="1"/>
       <c r="P52" s="1"/>
@@ -4671,21 +4676,21 @@
       <c r="Z52" s="1"/>
     </row>
     <row r="53" spans="1:26" ht="15.75">
-      <c r="A53" s="18">
+      <c r="A53" s="17">
         <v>42</v>
       </c>
-      <c r="B53" s="15"/>
-      <c r="C53" s="15"/>
-      <c r="D53" s="15"/>
-      <c r="E53" s="8"/>
-      <c r="F53" s="8"/>
-      <c r="G53" s="8"/>
-      <c r="H53" s="15"/>
-      <c r="I53" s="15"/>
-      <c r="J53" s="15"/>
-      <c r="K53" s="39"/>
-      <c r="L53" s="9"/>
-      <c r="M53" s="9"/>
+      <c r="B53" s="14"/>
+      <c r="C53" s="14"/>
+      <c r="D53" s="14"/>
+      <c r="E53" s="7"/>
+      <c r="F53" s="7"/>
+      <c r="G53" s="7"/>
+      <c r="H53" s="14"/>
+      <c r="I53" s="14"/>
+      <c r="J53" s="14"/>
+      <c r="K53" s="37"/>
+      <c r="L53" s="8"/>
+      <c r="M53" s="8"/>
       <c r="N53" s="1"/>
       <c r="O53" s="1"/>
       <c r="P53" s="1"/>
@@ -4701,21 +4706,21 @@
       <c r="Z53" s="1"/>
     </row>
     <row r="54" spans="1:26" ht="15.75">
-      <c r="A54" s="17">
+      <c r="A54" s="16">
         <v>43</v>
       </c>
-      <c r="B54" s="14"/>
-      <c r="C54" s="13"/>
-      <c r="D54" s="13"/>
-      <c r="E54" s="7"/>
-      <c r="F54" s="7"/>
-      <c r="G54" s="7"/>
-      <c r="H54" s="13"/>
-      <c r="I54" s="13"/>
-      <c r="J54" s="13"/>
-      <c r="K54" s="38"/>
-      <c r="L54" s="12"/>
-      <c r="M54" s="12"/>
+      <c r="B54" s="13"/>
+      <c r="C54" s="12"/>
+      <c r="D54" s="12"/>
+      <c r="E54" s="6"/>
+      <c r="F54" s="6"/>
+      <c r="G54" s="6"/>
+      <c r="H54" s="12"/>
+      <c r="I54" s="12"/>
+      <c r="J54" s="12"/>
+      <c r="K54" s="36"/>
+      <c r="L54" s="11"/>
+      <c r="M54" s="11"/>
       <c r="N54" s="1"/>
       <c r="O54" s="1"/>
       <c r="P54" s="1"/>
@@ -4731,21 +4736,21 @@
       <c r="Z54" s="1"/>
     </row>
     <row r="55" spans="1:26" ht="15.75">
-      <c r="A55" s="18">
+      <c r="A55" s="17">
         <v>44</v>
       </c>
-      <c r="B55" s="15"/>
-      <c r="C55" s="15"/>
-      <c r="D55" s="15"/>
-      <c r="E55" s="8"/>
-      <c r="F55" s="8"/>
-      <c r="G55" s="8"/>
-      <c r="H55" s="15"/>
-      <c r="I55" s="15"/>
-      <c r="J55" s="15"/>
-      <c r="K55" s="39"/>
-      <c r="L55" s="9"/>
-      <c r="M55" s="9"/>
+      <c r="B55" s="14"/>
+      <c r="C55" s="14"/>
+      <c r="D55" s="14"/>
+      <c r="E55" s="7"/>
+      <c r="F55" s="7"/>
+      <c r="G55" s="7"/>
+      <c r="H55" s="14"/>
+      <c r="I55" s="14"/>
+      <c r="J55" s="14"/>
+      <c r="K55" s="37"/>
+      <c r="L55" s="8"/>
+      <c r="M55" s="8"/>
       <c r="N55" s="1"/>
       <c r="O55" s="1"/>
       <c r="P55" s="1"/>
@@ -4761,21 +4766,21 @@
       <c r="Z55" s="1"/>
     </row>
     <row r="56" spans="1:26" ht="15.75">
-      <c r="A56" s="16">
+      <c r="A56" s="15">
         <v>45</v>
       </c>
-      <c r="B56" s="14"/>
-      <c r="C56" s="13"/>
-      <c r="D56" s="13"/>
-      <c r="E56" s="7"/>
-      <c r="F56" s="7"/>
-      <c r="G56" s="7"/>
-      <c r="H56" s="13"/>
-      <c r="I56" s="13"/>
-      <c r="J56" s="13"/>
-      <c r="K56" s="38"/>
-      <c r="L56" s="11"/>
-      <c r="M56" s="12"/>
+      <c r="B56" s="13"/>
+      <c r="C56" s="12"/>
+      <c r="D56" s="12"/>
+      <c r="E56" s="6"/>
+      <c r="F56" s="6"/>
+      <c r="G56" s="6"/>
+      <c r="H56" s="12"/>
+      <c r="I56" s="12"/>
+      <c r="J56" s="12"/>
+      <c r="K56" s="36"/>
+      <c r="L56" s="10"/>
+      <c r="M56" s="11"/>
       <c r="N56" s="1"/>
       <c r="O56" s="1"/>
       <c r="P56" s="1"/>
@@ -4791,21 +4796,21 @@
       <c r="Z56" s="1"/>
     </row>
     <row r="57" spans="1:26" ht="15.75">
-      <c r="A57" s="18">
+      <c r="A57" s="17">
         <v>46</v>
       </c>
-      <c r="B57" s="15"/>
-      <c r="C57" s="15"/>
-      <c r="D57" s="15"/>
-      <c r="E57" s="8"/>
-      <c r="F57" s="8"/>
-      <c r="G57" s="8"/>
-      <c r="H57" s="15"/>
-      <c r="I57" s="15"/>
-      <c r="J57" s="15"/>
-      <c r="K57" s="39"/>
-      <c r="L57" s="9"/>
-      <c r="M57" s="9"/>
+      <c r="B57" s="14"/>
+      <c r="C57" s="14"/>
+      <c r="D57" s="14"/>
+      <c r="E57" s="7"/>
+      <c r="F57" s="7"/>
+      <c r="G57" s="7"/>
+      <c r="H57" s="14"/>
+      <c r="I57" s="14"/>
+      <c r="J57" s="14"/>
+      <c r="K57" s="37"/>
+      <c r="L57" s="8"/>
+      <c r="M57" s="8"/>
       <c r="N57" s="1"/>
       <c r="O57" s="1"/>
       <c r="P57" s="1"/>
@@ -4821,21 +4826,21 @@
       <c r="Z57" s="1"/>
     </row>
     <row r="58" spans="1:26" ht="15.75">
-      <c r="A58" s="17">
+      <c r="A58" s="16">
         <v>47</v>
       </c>
-      <c r="B58" s="14"/>
-      <c r="C58" s="13"/>
-      <c r="D58" s="13"/>
-      <c r="E58" s="7"/>
-      <c r="F58" s="7"/>
-      <c r="G58" s="7"/>
-      <c r="H58" s="13"/>
-      <c r="I58" s="13"/>
-      <c r="J58" s="13"/>
-      <c r="K58" s="38"/>
-      <c r="L58" s="12"/>
-      <c r="M58" s="12"/>
+      <c r="B58" s="13"/>
+      <c r="C58" s="12"/>
+      <c r="D58" s="12"/>
+      <c r="E58" s="6"/>
+      <c r="F58" s="6"/>
+      <c r="G58" s="6"/>
+      <c r="H58" s="12"/>
+      <c r="I58" s="12"/>
+      <c r="J58" s="12"/>
+      <c r="K58" s="36"/>
+      <c r="L58" s="11"/>
+      <c r="M58" s="11"/>
       <c r="N58" s="1"/>
       <c r="O58" s="1"/>
       <c r="P58" s="1"/>
@@ -4851,21 +4856,21 @@
       <c r="Z58" s="1"/>
     </row>
     <row r="59" spans="1:26" ht="15.75">
-      <c r="A59" s="18">
+      <c r="A59" s="17">
         <v>48</v>
       </c>
-      <c r="B59" s="15"/>
-      <c r="C59" s="15"/>
-      <c r="D59" s="36"/>
-      <c r="E59" s="8"/>
-      <c r="F59" s="8"/>
-      <c r="G59" s="8"/>
-      <c r="H59" s="15"/>
-      <c r="I59" s="15"/>
-      <c r="J59" s="15"/>
-      <c r="K59" s="39"/>
-      <c r="L59" s="9"/>
-      <c r="M59" s="9"/>
+      <c r="B59" s="14"/>
+      <c r="C59" s="14"/>
+      <c r="D59" s="34"/>
+      <c r="E59" s="7"/>
+      <c r="F59" s="7"/>
+      <c r="G59" s="7"/>
+      <c r="H59" s="14"/>
+      <c r="I59" s="14"/>
+      <c r="J59" s="14"/>
+      <c r="K59" s="37"/>
+      <c r="L59" s="8"/>
+      <c r="M59" s="8"/>
       <c r="N59" s="1"/>
       <c r="O59" s="1"/>
       <c r="P59" s="1"/>
@@ -4881,21 +4886,21 @@
       <c r="Z59" s="1"/>
     </row>
     <row r="60" spans="1:26" ht="15.75">
-      <c r="A60" s="16">
+      <c r="A60" s="15">
         <v>49</v>
       </c>
-      <c r="B60" s="14"/>
-      <c r="C60" s="13"/>
-      <c r="D60" s="37"/>
-      <c r="E60" s="7"/>
-      <c r="F60" s="7"/>
-      <c r="G60" s="7"/>
-      <c r="H60" s="13"/>
-      <c r="I60" s="13"/>
-      <c r="J60" s="13"/>
-      <c r="K60" s="38"/>
-      <c r="L60" s="11"/>
-      <c r="M60" s="12"/>
+      <c r="B60" s="13"/>
+      <c r="C60" s="12"/>
+      <c r="D60" s="35"/>
+      <c r="E60" s="6"/>
+      <c r="F60" s="6"/>
+      <c r="G60" s="6"/>
+      <c r="H60" s="12"/>
+      <c r="I60" s="12"/>
+      <c r="J60" s="12"/>
+      <c r="K60" s="36"/>
+      <c r="L60" s="10"/>
+      <c r="M60" s="11"/>
       <c r="N60" s="1"/>
       <c r="O60" s="1"/>
       <c r="P60" s="1"/>
@@ -4911,21 +4916,21 @@
       <c r="Z60" s="1"/>
     </row>
     <row r="61" spans="1:26" ht="15.75">
-      <c r="A61" s="18">
+      <c r="A61" s="17">
         <v>50</v>
       </c>
-      <c r="B61" s="15"/>
-      <c r="C61" s="15"/>
-      <c r="D61" s="36"/>
-      <c r="E61" s="8"/>
-      <c r="F61" s="8"/>
-      <c r="G61" s="8"/>
-      <c r="H61" s="15"/>
-      <c r="I61" s="15"/>
-      <c r="J61" s="15"/>
-      <c r="K61" s="39"/>
-      <c r="L61" s="9"/>
-      <c r="M61" s="9"/>
+      <c r="B61" s="14"/>
+      <c r="C61" s="14"/>
+      <c r="D61" s="34"/>
+      <c r="E61" s="7"/>
+      <c r="F61" s="7"/>
+      <c r="G61" s="7"/>
+      <c r="H61" s="14"/>
+      <c r="I61" s="14"/>
+      <c r="J61" s="14"/>
+      <c r="K61" s="37"/>
+      <c r="L61" s="8"/>
+      <c r="M61" s="8"/>
       <c r="N61" s="1"/>
       <c r="O61" s="1"/>
       <c r="P61" s="1"/>
@@ -4941,21 +4946,21 @@
       <c r="Z61" s="1"/>
     </row>
     <row r="62" spans="1:26" ht="15.75">
-      <c r="A62" s="17">
+      <c r="A62" s="16">
         <v>51</v>
       </c>
-      <c r="B62" s="14"/>
-      <c r="C62" s="13"/>
-      <c r="D62" s="37"/>
-      <c r="E62" s="7"/>
-      <c r="F62" s="7"/>
-      <c r="G62" s="7"/>
-      <c r="H62" s="13"/>
-      <c r="I62" s="13"/>
-      <c r="J62" s="13"/>
-      <c r="K62" s="38"/>
-      <c r="L62" s="12"/>
-      <c r="M62" s="12"/>
+      <c r="B62" s="13"/>
+      <c r="C62" s="12"/>
+      <c r="D62" s="35"/>
+      <c r="E62" s="6"/>
+      <c r="F62" s="6"/>
+      <c r="G62" s="6"/>
+      <c r="H62" s="12"/>
+      <c r="I62" s="12"/>
+      <c r="J62" s="12"/>
+      <c r="K62" s="36"/>
+      <c r="L62" s="11"/>
+      <c r="M62" s="11"/>
       <c r="N62" s="1"/>
       <c r="O62" s="1"/>
       <c r="P62" s="1"/>
@@ -4971,21 +4976,21 @@
       <c r="Z62" s="1"/>
     </row>
     <row r="63" spans="1:26" ht="15.75">
-      <c r="A63" s="18">
+      <c r="A63" s="17">
         <v>52</v>
       </c>
-      <c r="B63" s="15"/>
-      <c r="C63" s="15"/>
-      <c r="D63" s="8"/>
-      <c r="E63" s="8"/>
-      <c r="F63" s="8"/>
-      <c r="G63" s="8"/>
-      <c r="H63" s="15"/>
-      <c r="I63" s="10"/>
-      <c r="J63" s="15"/>
-      <c r="K63" s="10"/>
-      <c r="L63" s="9"/>
-      <c r="M63" s="9"/>
+      <c r="B63" s="14"/>
+      <c r="C63" s="14"/>
+      <c r="D63" s="7"/>
+      <c r="E63" s="7"/>
+      <c r="F63" s="7"/>
+      <c r="G63" s="7"/>
+      <c r="H63" s="14"/>
+      <c r="I63" s="9"/>
+      <c r="J63" s="14"/>
+      <c r="K63" s="9"/>
+      <c r="L63" s="8"/>
+      <c r="M63" s="8"/>
       <c r="N63" s="1"/>
       <c r="O63" s="1"/>
       <c r="P63" s="1"/>
@@ -5001,21 +5006,21 @@
       <c r="Z63" s="1"/>
     </row>
     <row r="64" spans="1:26" ht="15.75">
-      <c r="A64" s="16">
+      <c r="A64" s="15">
         <v>53</v>
       </c>
-      <c r="B64" s="13"/>
-      <c r="C64" s="7"/>
-      <c r="D64" s="7"/>
-      <c r="E64" s="7"/>
-      <c r="F64" s="7"/>
-      <c r="G64" s="7"/>
-      <c r="H64" s="13"/>
-      <c r="I64" s="11"/>
-      <c r="J64" s="13"/>
-      <c r="K64" s="11"/>
-      <c r="L64" s="11"/>
-      <c r="M64" s="12"/>
+      <c r="B64" s="12"/>
+      <c r="C64" s="6"/>
+      <c r="D64" s="6"/>
+      <c r="E64" s="6"/>
+      <c r="F64" s="6"/>
+      <c r="G64" s="6"/>
+      <c r="H64" s="12"/>
+      <c r="I64" s="10"/>
+      <c r="J64" s="12"/>
+      <c r="K64" s="10"/>
+      <c r="L64" s="10"/>
+      <c r="M64" s="11"/>
       <c r="N64" s="1"/>
       <c r="O64" s="1"/>
       <c r="P64" s="1"/>
@@ -5031,21 +5036,21 @@
       <c r="Z64" s="1"/>
     </row>
     <row r="65" spans="1:26" ht="15.75">
-      <c r="A65" s="18">
+      <c r="A65" s="17">
         <v>54</v>
       </c>
-      <c r="B65" s="15"/>
-      <c r="C65" s="8"/>
-      <c r="D65" s="8"/>
-      <c r="E65" s="8"/>
-      <c r="F65" s="8"/>
-      <c r="G65" s="8"/>
-      <c r="H65" s="15"/>
-      <c r="I65" s="10"/>
-      <c r="J65" s="15"/>
-      <c r="K65" s="10"/>
-      <c r="L65" s="9"/>
-      <c r="M65" s="9"/>
+      <c r="B65" s="14"/>
+      <c r="C65" s="7"/>
+      <c r="D65" s="7"/>
+      <c r="E65" s="7"/>
+      <c r="F65" s="7"/>
+      <c r="G65" s="7"/>
+      <c r="H65" s="14"/>
+      <c r="I65" s="9"/>
+      <c r="J65" s="14"/>
+      <c r="K65" s="9"/>
+      <c r="L65" s="8"/>
+      <c r="M65" s="8"/>
       <c r="N65" s="1"/>
       <c r="O65" s="1"/>
       <c r="P65" s="1"/>
@@ -5061,21 +5066,21 @@
       <c r="Z65" s="1"/>
     </row>
     <row r="66" spans="1:26" ht="15.75">
-      <c r="A66" s="17">
+      <c r="A66" s="16">
         <v>55</v>
       </c>
-      <c r="B66" s="14"/>
-      <c r="C66" s="7"/>
-      <c r="D66" s="7"/>
-      <c r="E66" s="7"/>
-      <c r="F66" s="7"/>
-      <c r="G66" s="7"/>
-      <c r="H66" s="13"/>
-      <c r="I66" s="12"/>
-      <c r="J66" s="13"/>
-      <c r="K66" s="12"/>
-      <c r="L66" s="12"/>
-      <c r="M66" s="12"/>
+      <c r="B66" s="13"/>
+      <c r="C66" s="6"/>
+      <c r="D66" s="6"/>
+      <c r="E66" s="6"/>
+      <c r="F66" s="6"/>
+      <c r="G66" s="6"/>
+      <c r="H66" s="12"/>
+      <c r="I66" s="11"/>
+      <c r="J66" s="12"/>
+      <c r="K66" s="11"/>
+      <c r="L66" s="11"/>
+      <c r="M66" s="11"/>
       <c r="N66" s="1"/>
       <c r="O66" s="1"/>
       <c r="P66" s="1"/>
@@ -5091,21 +5096,21 @@
       <c r="Z66" s="1"/>
     </row>
     <row r="67" spans="1:26" ht="15.75">
-      <c r="A67" s="18">
+      <c r="A67" s="17">
         <v>56</v>
       </c>
-      <c r="B67" s="15"/>
-      <c r="C67" s="8"/>
-      <c r="D67" s="8"/>
-      <c r="E67" s="8"/>
-      <c r="F67" s="8"/>
-      <c r="G67" s="8"/>
-      <c r="H67" s="15"/>
-      <c r="I67" s="10"/>
-      <c r="J67" s="15"/>
-      <c r="K67" s="10"/>
-      <c r="L67" s="9"/>
-      <c r="M67" s="9"/>
+      <c r="B67" s="14"/>
+      <c r="C67" s="7"/>
+      <c r="D67" s="7"/>
+      <c r="E67" s="7"/>
+      <c r="F67" s="7"/>
+      <c r="G67" s="7"/>
+      <c r="H67" s="14"/>
+      <c r="I67" s="9"/>
+      <c r="J67" s="14"/>
+      <c r="K67" s="9"/>
+      <c r="L67" s="8"/>
+      <c r="M67" s="8"/>
       <c r="N67" s="1"/>
       <c r="O67" s="1"/>
       <c r="P67" s="1"/>
@@ -5121,21 +5126,21 @@
       <c r="Z67" s="1"/>
     </row>
     <row r="68" spans="1:26" ht="15.75">
-      <c r="A68" s="16">
+      <c r="A68" s="15">
         <v>57</v>
       </c>
-      <c r="B68" s="13"/>
-      <c r="C68" s="7"/>
-      <c r="D68" s="7"/>
-      <c r="E68" s="7"/>
-      <c r="F68" s="7"/>
-      <c r="G68" s="7"/>
-      <c r="H68" s="13"/>
-      <c r="I68" s="11"/>
-      <c r="J68" s="13"/>
-      <c r="K68" s="11"/>
-      <c r="L68" s="11"/>
-      <c r="M68" s="12"/>
+      <c r="B68" s="12"/>
+      <c r="C68" s="6"/>
+      <c r="D68" s="6"/>
+      <c r="E68" s="6"/>
+      <c r="F68" s="6"/>
+      <c r="G68" s="6"/>
+      <c r="H68" s="12"/>
+      <c r="I68" s="10"/>
+      <c r="J68" s="12"/>
+      <c r="K68" s="10"/>
+      <c r="L68" s="10"/>
+      <c r="M68" s="11"/>
       <c r="N68" s="1"/>
       <c r="O68" s="1"/>
       <c r="P68" s="1"/>
@@ -5151,21 +5156,21 @@
       <c r="Z68" s="1"/>
     </row>
     <row r="69" spans="1:26" ht="15.75">
-      <c r="A69" s="18">
+      <c r="A69" s="17">
         <v>58</v>
       </c>
-      <c r="B69" s="15"/>
-      <c r="C69" s="8"/>
-      <c r="D69" s="8"/>
-      <c r="E69" s="8"/>
-      <c r="F69" s="8"/>
-      <c r="G69" s="8"/>
-      <c r="H69" s="15"/>
-      <c r="I69" s="10"/>
-      <c r="J69" s="15"/>
-      <c r="K69" s="10"/>
-      <c r="L69" s="9"/>
-      <c r="M69" s="9"/>
+      <c r="B69" s="14"/>
+      <c r="C69" s="7"/>
+      <c r="D69" s="7"/>
+      <c r="E69" s="7"/>
+      <c r="F69" s="7"/>
+      <c r="G69" s="7"/>
+      <c r="H69" s="14"/>
+      <c r="I69" s="9"/>
+      <c r="J69" s="14"/>
+      <c r="K69" s="9"/>
+      <c r="L69" s="8"/>
+      <c r="M69" s="8"/>
       <c r="N69" s="1"/>
       <c r="O69" s="1"/>
       <c r="P69" s="1"/>
@@ -5181,21 +5186,21 @@
       <c r="Z69" s="1"/>
     </row>
     <row r="70" spans="1:26" ht="15.75">
-      <c r="A70" s="17">
+      <c r="A70" s="16">
         <v>59</v>
       </c>
-      <c r="B70" s="14"/>
-      <c r="C70" s="7"/>
-      <c r="D70" s="7"/>
-      <c r="E70" s="7"/>
-      <c r="F70" s="7"/>
-      <c r="G70" s="7"/>
-      <c r="H70" s="13"/>
-      <c r="I70" s="12"/>
-      <c r="J70" s="13"/>
-      <c r="K70" s="12"/>
-      <c r="L70" s="12"/>
-      <c r="M70" s="12"/>
+      <c r="B70" s="13"/>
+      <c r="C70" s="6"/>
+      <c r="D70" s="6"/>
+      <c r="E70" s="6"/>
+      <c r="F70" s="6"/>
+      <c r="G70" s="6"/>
+      <c r="H70" s="12"/>
+      <c r="I70" s="11"/>
+      <c r="J70" s="12"/>
+      <c r="K70" s="11"/>
+      <c r="L70" s="11"/>
+      <c r="M70" s="11"/>
       <c r="N70" s="1"/>
       <c r="O70" s="1"/>
       <c r="P70" s="1"/>
@@ -5211,21 +5216,21 @@
       <c r="Z70" s="1"/>
     </row>
     <row r="71" spans="1:26" ht="15.75">
-      <c r="A71" s="18">
+      <c r="A71" s="17">
         <v>60</v>
       </c>
-      <c r="B71" s="15"/>
-      <c r="C71" s="8"/>
-      <c r="D71" s="8"/>
-      <c r="E71" s="8"/>
-      <c r="F71" s="8"/>
-      <c r="G71" s="8"/>
-      <c r="H71" s="15"/>
-      <c r="I71" s="10"/>
-      <c r="J71" s="15"/>
-      <c r="K71" s="10"/>
-      <c r="L71" s="9"/>
-      <c r="M71" s="9"/>
+      <c r="B71" s="14"/>
+      <c r="C71" s="7"/>
+      <c r="D71" s="7"/>
+      <c r="E71" s="7"/>
+      <c r="F71" s="7"/>
+      <c r="G71" s="7"/>
+      <c r="H71" s="14"/>
+      <c r="I71" s="9"/>
+      <c r="J71" s="14"/>
+      <c r="K71" s="9"/>
+      <c r="L71" s="8"/>
+      <c r="M71" s="8"/>
       <c r="N71" s="1"/>
       <c r="O71" s="1"/>
       <c r="P71" s="1"/>
@@ -5241,21 +5246,21 @@
       <c r="Z71" s="1"/>
     </row>
     <row r="72" spans="1:26" ht="15.75">
-      <c r="A72" s="16">
+      <c r="A72" s="15">
         <v>61</v>
       </c>
-      <c r="B72" s="13"/>
-      <c r="C72" s="7"/>
-      <c r="D72" s="7"/>
-      <c r="E72" s="7"/>
-      <c r="F72" s="7"/>
-      <c r="G72" s="7"/>
-      <c r="H72" s="13"/>
-      <c r="I72" s="11"/>
-      <c r="J72" s="13"/>
-      <c r="K72" s="11"/>
-      <c r="L72" s="11"/>
-      <c r="M72" s="12"/>
+      <c r="B72" s="12"/>
+      <c r="C72" s="6"/>
+      <c r="D72" s="6"/>
+      <c r="E72" s="6"/>
+      <c r="F72" s="6"/>
+      <c r="G72" s="6"/>
+      <c r="H72" s="12"/>
+      <c r="I72" s="10"/>
+      <c r="J72" s="12"/>
+      <c r="K72" s="10"/>
+      <c r="L72" s="10"/>
+      <c r="M72" s="11"/>
       <c r="N72" s="1"/>
       <c r="O72" s="1"/>
       <c r="P72" s="1"/>
@@ -5271,21 +5276,21 @@
       <c r="Z72" s="1"/>
     </row>
     <row r="73" spans="1:26" ht="15.75">
-      <c r="A73" s="18">
+      <c r="A73" s="17">
         <v>62</v>
       </c>
-      <c r="B73" s="15"/>
-      <c r="C73" s="8"/>
-      <c r="D73" s="8"/>
-      <c r="E73" s="8"/>
-      <c r="F73" s="8"/>
-      <c r="G73" s="8"/>
-      <c r="H73" s="15"/>
-      <c r="I73" s="10"/>
-      <c r="J73" s="15"/>
-      <c r="K73" s="10"/>
-      <c r="L73" s="9"/>
-      <c r="M73" s="9"/>
+      <c r="B73" s="14"/>
+      <c r="C73" s="7"/>
+      <c r="D73" s="7"/>
+      <c r="E73" s="7"/>
+      <c r="F73" s="7"/>
+      <c r="G73" s="7"/>
+      <c r="H73" s="14"/>
+      <c r="I73" s="9"/>
+      <c r="J73" s="14"/>
+      <c r="K73" s="9"/>
+      <c r="L73" s="8"/>
+      <c r="M73" s="8"/>
       <c r="N73" s="1"/>
       <c r="O73" s="1"/>
       <c r="P73" s="1"/>
@@ -5301,21 +5306,21 @@
       <c r="Z73" s="1"/>
     </row>
     <row r="74" spans="1:26" ht="15.75">
-      <c r="A74" s="17">
+      <c r="A74" s="16">
         <v>63</v>
       </c>
-      <c r="B74" s="14"/>
-      <c r="C74" s="7"/>
-      <c r="D74" s="7"/>
-      <c r="E74" s="7"/>
-      <c r="F74" s="7"/>
-      <c r="G74" s="7"/>
-      <c r="H74" s="13"/>
-      <c r="I74" s="12"/>
-      <c r="J74" s="13"/>
-      <c r="K74" s="12"/>
-      <c r="L74" s="12"/>
-      <c r="M74" s="12"/>
+      <c r="B74" s="13"/>
+      <c r="C74" s="6"/>
+      <c r="D74" s="6"/>
+      <c r="E74" s="6"/>
+      <c r="F74" s="6"/>
+      <c r="G74" s="6"/>
+      <c r="H74" s="12"/>
+      <c r="I74" s="11"/>
+      <c r="J74" s="12"/>
+      <c r="K74" s="11"/>
+      <c r="L74" s="11"/>
+      <c r="M74" s="11"/>
       <c r="N74" s="1"/>
       <c r="O74" s="1"/>
       <c r="P74" s="1"/>
@@ -5331,21 +5336,21 @@
       <c r="Z74" s="1"/>
     </row>
     <row r="75" spans="1:26" ht="15.75">
-      <c r="A75" s="18">
+      <c r="A75" s="17">
         <v>64</v>
       </c>
-      <c r="B75" s="15"/>
-      <c r="C75" s="8"/>
-      <c r="D75" s="8"/>
-      <c r="E75" s="8"/>
-      <c r="F75" s="8"/>
-      <c r="G75" s="8"/>
-      <c r="H75" s="15"/>
-      <c r="I75" s="10"/>
-      <c r="J75" s="15"/>
-      <c r="K75" s="10"/>
-      <c r="L75" s="9"/>
-      <c r="M75" s="9"/>
+      <c r="B75" s="14"/>
+      <c r="C75" s="7"/>
+      <c r="D75" s="7"/>
+      <c r="E75" s="7"/>
+      <c r="F75" s="7"/>
+      <c r="G75" s="7"/>
+      <c r="H75" s="14"/>
+      <c r="I75" s="9"/>
+      <c r="J75" s="14"/>
+      <c r="K75" s="9"/>
+      <c r="L75" s="8"/>
+      <c r="M75" s="8"/>
       <c r="N75" s="1"/>
       <c r="O75" s="1"/>
       <c r="P75" s="1"/>
@@ -5361,21 +5366,21 @@
       <c r="Z75" s="1"/>
     </row>
     <row r="76" spans="1:26" ht="15.75">
-      <c r="A76" s="16">
+      <c r="A76" s="15">
         <v>65</v>
       </c>
-      <c r="B76" s="13"/>
-      <c r="C76" s="7"/>
-      <c r="D76" s="7"/>
-      <c r="E76" s="7"/>
-      <c r="F76" s="7"/>
-      <c r="G76" s="7"/>
-      <c r="H76" s="13"/>
-      <c r="I76" s="11"/>
-      <c r="J76" s="13"/>
-      <c r="K76" s="11"/>
-      <c r="L76" s="11"/>
-      <c r="M76" s="12"/>
+      <c r="B76" s="12"/>
+      <c r="C76" s="6"/>
+      <c r="D76" s="6"/>
+      <c r="E76" s="6"/>
+      <c r="F76" s="6"/>
+      <c r="G76" s="6"/>
+      <c r="H76" s="12"/>
+      <c r="I76" s="10"/>
+      <c r="J76" s="12"/>
+      <c r="K76" s="10"/>
+      <c r="L76" s="10"/>
+      <c r="M76" s="11"/>
       <c r="N76" s="1"/>
       <c r="O76" s="1"/>
       <c r="P76" s="1"/>
@@ -5391,21 +5396,21 @@
       <c r="Z76" s="1"/>
     </row>
     <row r="77" spans="1:26" ht="15.75">
-      <c r="A77" s="18">
+      <c r="A77" s="17">
         <v>66</v>
       </c>
-      <c r="B77" s="15"/>
-      <c r="C77" s="8"/>
-      <c r="D77" s="8"/>
-      <c r="E77" s="8"/>
-      <c r="F77" s="8"/>
-      <c r="G77" s="8"/>
-      <c r="H77" s="15"/>
-      <c r="I77" s="10"/>
-      <c r="J77" s="15"/>
-      <c r="K77" s="10"/>
-      <c r="L77" s="9"/>
-      <c r="M77" s="9"/>
+      <c r="B77" s="14"/>
+      <c r="C77" s="7"/>
+      <c r="D77" s="7"/>
+      <c r="E77" s="7"/>
+      <c r="F77" s="7"/>
+      <c r="G77" s="7"/>
+      <c r="H77" s="14"/>
+      <c r="I77" s="9"/>
+      <c r="J77" s="14"/>
+      <c r="K77" s="9"/>
+      <c r="L77" s="8"/>
+      <c r="M77" s="8"/>
       <c r="N77" s="1"/>
       <c r="O77" s="1"/>
       <c r="P77" s="1"/>
@@ -5421,21 +5426,21 @@
       <c r="Z77" s="1"/>
     </row>
     <row r="78" spans="1:26" ht="15.75">
-      <c r="A78" s="17">
+      <c r="A78" s="16">
         <v>67</v>
       </c>
-      <c r="B78" s="14"/>
-      <c r="C78" s="7"/>
-      <c r="D78" s="7"/>
-      <c r="E78" s="7"/>
-      <c r="F78" s="7"/>
-      <c r="G78" s="7"/>
-      <c r="H78" s="13"/>
-      <c r="I78" s="12"/>
-      <c r="J78" s="13"/>
-      <c r="K78" s="12"/>
-      <c r="L78" s="12"/>
-      <c r="M78" s="12"/>
+      <c r="B78" s="13"/>
+      <c r="C78" s="6"/>
+      <c r="D78" s="6"/>
+      <c r="E78" s="6"/>
+      <c r="F78" s="6"/>
+      <c r="G78" s="6"/>
+      <c r="H78" s="12"/>
+      <c r="I78" s="11"/>
+      <c r="J78" s="12"/>
+      <c r="K78" s="11"/>
+      <c r="L78" s="11"/>
+      <c r="M78" s="11"/>
       <c r="N78" s="1"/>
       <c r="O78" s="1"/>
       <c r="P78" s="1"/>
@@ -5451,21 +5456,21 @@
       <c r="Z78" s="1"/>
     </row>
     <row r="79" spans="1:26" ht="15.75">
-      <c r="A79" s="18">
+      <c r="A79" s="17">
         <v>68</v>
       </c>
-      <c r="B79" s="15"/>
-      <c r="C79" s="8"/>
-      <c r="D79" s="8"/>
-      <c r="E79" s="8"/>
-      <c r="F79" s="8"/>
-      <c r="G79" s="8"/>
-      <c r="H79" s="15"/>
-      <c r="I79" s="10"/>
-      <c r="J79" s="15"/>
-      <c r="K79" s="10"/>
-      <c r="L79" s="9"/>
-      <c r="M79" s="9"/>
+      <c r="B79" s="14"/>
+      <c r="C79" s="7"/>
+      <c r="D79" s="7"/>
+      <c r="E79" s="7"/>
+      <c r="F79" s="7"/>
+      <c r="G79" s="7"/>
+      <c r="H79" s="14"/>
+      <c r="I79" s="9"/>
+      <c r="J79" s="14"/>
+      <c r="K79" s="9"/>
+      <c r="L79" s="8"/>
+      <c r="M79" s="8"/>
       <c r="N79" s="1"/>
       <c r="O79" s="1"/>
       <c r="P79" s="1"/>
@@ -5481,21 +5486,21 @@
       <c r="Z79" s="1"/>
     </row>
     <row r="80" spans="1:26" ht="15.75">
-      <c r="A80" s="16">
+      <c r="A80" s="15">
         <v>69</v>
       </c>
-      <c r="B80" s="13"/>
-      <c r="C80" s="7"/>
-      <c r="D80" s="7"/>
-      <c r="E80" s="7"/>
-      <c r="F80" s="7"/>
-      <c r="G80" s="7"/>
-      <c r="H80" s="13"/>
-      <c r="I80" s="11"/>
-      <c r="J80" s="13"/>
-      <c r="K80" s="11"/>
-      <c r="L80" s="11"/>
-      <c r="M80" s="12"/>
+      <c r="B80" s="12"/>
+      <c r="C80" s="6"/>
+      <c r="D80" s="6"/>
+      <c r="E80" s="6"/>
+      <c r="F80" s="6"/>
+      <c r="G80" s="6"/>
+      <c r="H80" s="12"/>
+      <c r="I80" s="10"/>
+      <c r="J80" s="12"/>
+      <c r="K80" s="10"/>
+      <c r="L80" s="10"/>
+      <c r="M80" s="11"/>
       <c r="N80" s="1"/>
       <c r="O80" s="1"/>
       <c r="P80" s="1"/>
@@ -5511,21 +5516,21 @@
       <c r="Z80" s="1"/>
     </row>
     <row r="81" spans="1:26" ht="15.75">
-      <c r="A81" s="18">
+      <c r="A81" s="17">
         <v>70</v>
       </c>
-      <c r="B81" s="15"/>
-      <c r="C81" s="8"/>
-      <c r="D81" s="8"/>
-      <c r="E81" s="8"/>
-      <c r="F81" s="8"/>
-      <c r="G81" s="8"/>
-      <c r="H81" s="15"/>
-      <c r="I81" s="10"/>
-      <c r="J81" s="15"/>
-      <c r="K81" s="10"/>
-      <c r="L81" s="9"/>
-      <c r="M81" s="9"/>
+      <c r="B81" s="14"/>
+      <c r="C81" s="7"/>
+      <c r="D81" s="7"/>
+      <c r="E81" s="7"/>
+      <c r="F81" s="7"/>
+      <c r="G81" s="7"/>
+      <c r="H81" s="14"/>
+      <c r="I81" s="9"/>
+      <c r="J81" s="14"/>
+      <c r="K81" s="9"/>
+      <c r="L81" s="8"/>
+      <c r="M81" s="8"/>
       <c r="N81" s="1"/>
       <c r="O81" s="1"/>
       <c r="P81" s="1"/>
@@ -5541,21 +5546,21 @@
       <c r="Z81" s="1"/>
     </row>
     <row r="82" spans="1:26" ht="15.75">
-      <c r="A82" s="17">
+      <c r="A82" s="16">
         <v>71</v>
       </c>
-      <c r="B82" s="14"/>
-      <c r="C82" s="7"/>
-      <c r="D82" s="7"/>
-      <c r="E82" s="7"/>
-      <c r="F82" s="7"/>
-      <c r="G82" s="7"/>
-      <c r="H82" s="13"/>
-      <c r="I82" s="12"/>
-      <c r="J82" s="13"/>
-      <c r="K82" s="12"/>
-      <c r="L82" s="12"/>
-      <c r="M82" s="12"/>
+      <c r="B82" s="13"/>
+      <c r="C82" s="6"/>
+      <c r="D82" s="6"/>
+      <c r="E82" s="6"/>
+      <c r="F82" s="6"/>
+      <c r="G82" s="6"/>
+      <c r="H82" s="12"/>
+      <c r="I82" s="11"/>
+      <c r="J82" s="12"/>
+      <c r="K82" s="11"/>
+      <c r="L82" s="11"/>
+      <c r="M82" s="11"/>
       <c r="N82" s="1"/>
       <c r="O82" s="1"/>
       <c r="P82" s="1"/>
@@ -5571,21 +5576,21 @@
       <c r="Z82" s="1"/>
     </row>
     <row r="83" spans="1:26" ht="15.75">
-      <c r="A83" s="18">
+      <c r="A83" s="17">
         <v>72</v>
       </c>
-      <c r="B83" s="15"/>
-      <c r="C83" s="8"/>
-      <c r="D83" s="8"/>
-      <c r="E83" s="8"/>
-      <c r="F83" s="8"/>
-      <c r="G83" s="8"/>
-      <c r="H83" s="15"/>
-      <c r="I83" s="10"/>
-      <c r="J83" s="15"/>
-      <c r="K83" s="10"/>
-      <c r="L83" s="9"/>
-      <c r="M83" s="9"/>
+      <c r="B83" s="14"/>
+      <c r="C83" s="7"/>
+      <c r="D83" s="7"/>
+      <c r="E83" s="7"/>
+      <c r="F83" s="7"/>
+      <c r="G83" s="7"/>
+      <c r="H83" s="14"/>
+      <c r="I83" s="9"/>
+      <c r="J83" s="14"/>
+      <c r="K83" s="9"/>
+      <c r="L83" s="8"/>
+      <c r="M83" s="8"/>
       <c r="N83" s="1"/>
       <c r="O83" s="1"/>
       <c r="P83" s="1"/>
@@ -5601,21 +5606,21 @@
       <c r="Z83" s="1"/>
     </row>
     <row r="84" spans="1:26" ht="15.75">
-      <c r="A84" s="16">
+      <c r="A84" s="15">
         <v>73</v>
       </c>
-      <c r="B84" s="13"/>
-      <c r="C84" s="7"/>
-      <c r="D84" s="7"/>
-      <c r="E84" s="7"/>
-      <c r="F84" s="7"/>
-      <c r="G84" s="7"/>
-      <c r="H84" s="13"/>
-      <c r="I84" s="11"/>
-      <c r="J84" s="13"/>
-      <c r="K84" s="11"/>
-      <c r="L84" s="11"/>
-      <c r="M84" s="12"/>
+      <c r="B84" s="12"/>
+      <c r="C84" s="6"/>
+      <c r="D84" s="6"/>
+      <c r="E84" s="6"/>
+      <c r="F84" s="6"/>
+      <c r="G84" s="6"/>
+      <c r="H84" s="12"/>
+      <c r="I84" s="10"/>
+      <c r="J84" s="12"/>
+      <c r="K84" s="10"/>
+      <c r="L84" s="10"/>
+      <c r="M84" s="11"/>
       <c r="N84" s="1"/>
       <c r="O84" s="1"/>
       <c r="P84" s="1"/>
@@ -5631,21 +5636,21 @@
       <c r="Z84" s="1"/>
     </row>
     <row r="85" spans="1:26" ht="15.75">
-      <c r="A85" s="18">
+      <c r="A85" s="17">
         <v>74</v>
       </c>
-      <c r="B85" s="15"/>
-      <c r="C85" s="8"/>
-      <c r="D85" s="8"/>
-      <c r="E85" s="8"/>
-      <c r="F85" s="8"/>
-      <c r="G85" s="8"/>
-      <c r="H85" s="15"/>
-      <c r="I85" s="10"/>
-      <c r="J85" s="15"/>
-      <c r="K85" s="10"/>
-      <c r="L85" s="9"/>
-      <c r="M85" s="9"/>
+      <c r="B85" s="14"/>
+      <c r="C85" s="7"/>
+      <c r="D85" s="7"/>
+      <c r="E85" s="7"/>
+      <c r="F85" s="7"/>
+      <c r="G85" s="7"/>
+      <c r="H85" s="14"/>
+      <c r="I85" s="9"/>
+      <c r="J85" s="14"/>
+      <c r="K85" s="9"/>
+      <c r="L85" s="8"/>
+      <c r="M85" s="8"/>
       <c r="N85" s="1"/>
       <c r="O85" s="1"/>
       <c r="P85" s="1"/>
@@ -5661,21 +5666,21 @@
       <c r="Z85" s="1"/>
     </row>
     <row r="86" spans="1:26" ht="15.75">
-      <c r="A86" s="16">
+      <c r="A86" s="15">
         <v>75</v>
       </c>
-      <c r="B86" s="14"/>
-      <c r="C86" s="7"/>
-      <c r="D86" s="7"/>
-      <c r="E86" s="7"/>
-      <c r="F86" s="7"/>
-      <c r="G86" s="7"/>
-      <c r="H86" s="13"/>
-      <c r="I86" s="12"/>
-      <c r="J86" s="13"/>
-      <c r="K86" s="12"/>
-      <c r="L86" s="12"/>
-      <c r="M86" s="12"/>
+      <c r="B86" s="13"/>
+      <c r="C86" s="6"/>
+      <c r="D86" s="6"/>
+      <c r="E86" s="6"/>
+      <c r="F86" s="6"/>
+      <c r="G86" s="6"/>
+      <c r="H86" s="12"/>
+      <c r="I86" s="11"/>
+      <c r="J86" s="12"/>
+      <c r="K86" s="11"/>
+      <c r="L86" s="11"/>
+      <c r="M86" s="11"/>
       <c r="N86" s="1"/>
       <c r="O86" s="1"/>
       <c r="P86" s="1"/>
@@ -5691,21 +5696,21 @@
       <c r="Z86" s="1"/>
     </row>
     <row r="87" spans="1:26" ht="15.75">
-      <c r="A87" s="18">
+      <c r="A87" s="17">
         <v>76</v>
       </c>
-      <c r="B87" s="15"/>
-      <c r="C87" s="15"/>
-      <c r="D87" s="15"/>
-      <c r="E87" s="15"/>
-      <c r="F87" s="15"/>
-      <c r="G87" s="8"/>
-      <c r="H87" s="15"/>
-      <c r="I87" s="10"/>
-      <c r="J87" s="15"/>
-      <c r="K87" s="10"/>
-      <c r="L87" s="9"/>
-      <c r="M87" s="9"/>
+      <c r="B87" s="14"/>
+      <c r="C87" s="14"/>
+      <c r="D87" s="14"/>
+      <c r="E87" s="14"/>
+      <c r="F87" s="14"/>
+      <c r="G87" s="7"/>
+      <c r="H87" s="14"/>
+      <c r="I87" s="9"/>
+      <c r="J87" s="14"/>
+      <c r="K87" s="9"/>
+      <c r="L87" s="8"/>
+      <c r="M87" s="8"/>
       <c r="N87" s="1"/>
       <c r="O87" s="1"/>
       <c r="P87" s="1"/>
@@ -5721,21 +5726,21 @@
       <c r="Z87" s="1"/>
     </row>
     <row r="88" spans="1:26" ht="15.75">
-      <c r="A88" s="16">
+      <c r="A88" s="15">
         <v>77</v>
       </c>
-      <c r="B88" s="14"/>
-      <c r="C88" s="14"/>
-      <c r="D88" s="14"/>
-      <c r="E88" s="14"/>
-      <c r="F88" s="14"/>
-      <c r="G88" s="7"/>
-      <c r="H88" s="13"/>
-      <c r="I88" s="12"/>
-      <c r="J88" s="13"/>
-      <c r="K88" s="12"/>
-      <c r="L88" s="12"/>
-      <c r="M88" s="12"/>
+      <c r="B88" s="13"/>
+      <c r="C88" s="13"/>
+      <c r="D88" s="13"/>
+      <c r="E88" s="13"/>
+      <c r="F88" s="13"/>
+      <c r="G88" s="6"/>
+      <c r="H88" s="12"/>
+      <c r="I88" s="11"/>
+      <c r="J88" s="12"/>
+      <c r="K88" s="11"/>
+      <c r="L88" s="11"/>
+      <c r="M88" s="11"/>
       <c r="N88" s="1"/>
       <c r="O88" s="1"/>
       <c r="P88" s="1"/>
@@ -5751,21 +5756,21 @@
       <c r="Z88" s="1"/>
     </row>
     <row r="89" spans="1:26" ht="15.75">
-      <c r="A89" s="18">
+      <c r="A89" s="17">
         <v>78</v>
       </c>
-      <c r="B89" s="15"/>
-      <c r="C89" s="15"/>
-      <c r="D89" s="15"/>
-      <c r="E89" s="15"/>
-      <c r="F89" s="15"/>
-      <c r="G89" s="8"/>
-      <c r="H89" s="15"/>
-      <c r="I89" s="10"/>
-      <c r="J89" s="15"/>
-      <c r="K89" s="10"/>
-      <c r="L89" s="9"/>
-      <c r="M89" s="9"/>
+      <c r="B89" s="14"/>
+      <c r="C89" s="14"/>
+      <c r="D89" s="14"/>
+      <c r="E89" s="14"/>
+      <c r="F89" s="14"/>
+      <c r="G89" s="7"/>
+      <c r="H89" s="14"/>
+      <c r="I89" s="9"/>
+      <c r="J89" s="14"/>
+      <c r="K89" s="9"/>
+      <c r="L89" s="8"/>
+      <c r="M89" s="8"/>
       <c r="N89" s="1"/>
       <c r="O89" s="1"/>
       <c r="P89" s="1"/>
@@ -5781,21 +5786,21 @@
       <c r="Z89" s="1"/>
     </row>
     <row r="90" spans="1:26" ht="15.75">
-      <c r="A90" s="16">
+      <c r="A90" s="15">
         <v>79</v>
       </c>
-      <c r="B90" s="14"/>
-      <c r="C90" s="14"/>
-      <c r="D90" s="14"/>
-      <c r="E90" s="14"/>
-      <c r="F90" s="14"/>
-      <c r="G90" s="7"/>
-      <c r="H90" s="13"/>
-      <c r="I90" s="12"/>
-      <c r="J90" s="13"/>
-      <c r="K90" s="12"/>
-      <c r="L90" s="12"/>
-      <c r="M90" s="12"/>
+      <c r="B90" s="13"/>
+      <c r="C90" s="13"/>
+      <c r="D90" s="13"/>
+      <c r="E90" s="13"/>
+      <c r="F90" s="13"/>
+      <c r="G90" s="6"/>
+      <c r="H90" s="12"/>
+      <c r="I90" s="11"/>
+      <c r="J90" s="12"/>
+      <c r="K90" s="11"/>
+      <c r="L90" s="11"/>
+      <c r="M90" s="11"/>
       <c r="N90" s="1"/>
       <c r="O90" s="1"/>
       <c r="P90" s="1"/>
@@ -5811,21 +5816,21 @@
       <c r="Z90" s="1"/>
     </row>
     <row r="91" spans="1:26" ht="15.75">
-      <c r="A91" s="18">
+      <c r="A91" s="17">
         <v>80</v>
       </c>
-      <c r="B91" s="15"/>
-      <c r="C91" s="15"/>
-      <c r="D91" s="15"/>
-      <c r="E91" s="15"/>
-      <c r="F91" s="15"/>
-      <c r="G91" s="8"/>
-      <c r="H91" s="15"/>
-      <c r="I91" s="10"/>
-      <c r="J91" s="15"/>
-      <c r="K91" s="10"/>
-      <c r="L91" s="9"/>
-      <c r="M91" s="9"/>
+      <c r="B91" s="14"/>
+      <c r="C91" s="14"/>
+      <c r="D91" s="14"/>
+      <c r="E91" s="14"/>
+      <c r="F91" s="14"/>
+      <c r="G91" s="7"/>
+      <c r="H91" s="14"/>
+      <c r="I91" s="9"/>
+      <c r="J91" s="14"/>
+      <c r="K91" s="9"/>
+      <c r="L91" s="8"/>
+      <c r="M91" s="8"/>
       <c r="N91" s="1"/>
       <c r="O91" s="1"/>
       <c r="P91" s="1"/>
@@ -5841,21 +5846,21 @@
       <c r="Z91" s="1"/>
     </row>
     <row r="92" spans="1:26" ht="15.75">
-      <c r="A92" s="16">
+      <c r="A92" s="15">
         <v>81</v>
       </c>
-      <c r="B92" s="14"/>
-      <c r="C92" s="14"/>
-      <c r="D92" s="14"/>
-      <c r="E92" s="14"/>
-      <c r="F92" s="14"/>
-      <c r="G92" s="7"/>
-      <c r="H92" s="13"/>
-      <c r="I92" s="12"/>
-      <c r="J92" s="13"/>
-      <c r="K92" s="12"/>
-      <c r="L92" s="12"/>
-      <c r="M92" s="12"/>
+      <c r="B92" s="13"/>
+      <c r="C92" s="13"/>
+      <c r="D92" s="13"/>
+      <c r="E92" s="13"/>
+      <c r="F92" s="13"/>
+      <c r="G92" s="6"/>
+      <c r="H92" s="12"/>
+      <c r="I92" s="11"/>
+      <c r="J92" s="12"/>
+      <c r="K92" s="11"/>
+      <c r="L92" s="11"/>
+      <c r="M92" s="11"/>
       <c r="N92" s="1"/>
       <c r="O92" s="1"/>
       <c r="P92" s="1"/>
@@ -5871,21 +5876,21 @@
       <c r="Z92" s="1"/>
     </row>
     <row r="93" spans="1:26" ht="15.75">
-      <c r="A93" s="18">
+      <c r="A93" s="17">
         <v>82</v>
       </c>
-      <c r="B93" s="15"/>
-      <c r="C93" s="15"/>
-      <c r="D93" s="15"/>
-      <c r="E93" s="15"/>
-      <c r="F93" s="15"/>
-      <c r="G93" s="8"/>
-      <c r="H93" s="15"/>
-      <c r="I93" s="10"/>
-      <c r="J93" s="15"/>
-      <c r="K93" s="10"/>
-      <c r="L93" s="9"/>
-      <c r="M93" s="9"/>
+      <c r="B93" s="14"/>
+      <c r="C93" s="14"/>
+      <c r="D93" s="14"/>
+      <c r="E93" s="14"/>
+      <c r="F93" s="14"/>
+      <c r="G93" s="7"/>
+      <c r="H93" s="14"/>
+      <c r="I93" s="9"/>
+      <c r="J93" s="14"/>
+      <c r="K93" s="9"/>
+      <c r="L93" s="8"/>
+      <c r="M93" s="8"/>
       <c r="N93" s="1"/>
       <c r="O93" s="1"/>
       <c r="P93" s="1"/>
@@ -5901,21 +5906,21 @@
       <c r="Z93" s="1"/>
     </row>
     <row r="94" spans="1:26" ht="15.75">
-      <c r="A94" s="16">
+      <c r="A94" s="15">
         <v>83</v>
       </c>
-      <c r="B94" s="14"/>
-      <c r="C94" s="14"/>
-      <c r="D94" s="14"/>
-      <c r="E94" s="14"/>
-      <c r="F94" s="14"/>
-      <c r="G94" s="7"/>
-      <c r="H94" s="13"/>
-      <c r="I94" s="12"/>
-      <c r="J94" s="13"/>
-      <c r="K94" s="12"/>
-      <c r="L94" s="12"/>
-      <c r="M94" s="12"/>
+      <c r="B94" s="13"/>
+      <c r="C94" s="13"/>
+      <c r="D94" s="13"/>
+      <c r="E94" s="13"/>
+      <c r="F94" s="13"/>
+      <c r="G94" s="6"/>
+      <c r="H94" s="12"/>
+      <c r="I94" s="11"/>
+      <c r="J94" s="12"/>
+      <c r="K94" s="11"/>
+      <c r="L94" s="11"/>
+      <c r="M94" s="11"/>
       <c r="N94" s="1"/>
       <c r="O94" s="1"/>
       <c r="P94" s="1"/>
@@ -5931,21 +5936,21 @@
       <c r="Z94" s="1"/>
     </row>
     <row r="95" spans="1:26" ht="15.75">
-      <c r="A95" s="18">
+      <c r="A95" s="17">
         <v>84</v>
       </c>
-      <c r="B95" s="15"/>
-      <c r="C95" s="15"/>
-      <c r="D95" s="15"/>
-      <c r="E95" s="15"/>
-      <c r="F95" s="15"/>
-      <c r="G95" s="8"/>
-      <c r="H95" s="15"/>
-      <c r="I95" s="10"/>
-      <c r="J95" s="15"/>
-      <c r="K95" s="10"/>
-      <c r="L95" s="9"/>
-      <c r="M95" s="9"/>
+      <c r="B95" s="14"/>
+      <c r="C95" s="14"/>
+      <c r="D95" s="14"/>
+      <c r="E95" s="14"/>
+      <c r="F95" s="14"/>
+      <c r="G95" s="7"/>
+      <c r="H95" s="14"/>
+      <c r="I95" s="9"/>
+      <c r="J95" s="14"/>
+      <c r="K95" s="9"/>
+      <c r="L95" s="8"/>
+      <c r="M95" s="8"/>
       <c r="N95" s="1"/>
       <c r="O95" s="1"/>
       <c r="P95" s="1"/>
@@ -5961,21 +5966,21 @@
       <c r="Z95" s="1"/>
     </row>
     <row r="96" spans="1:26" ht="15.75">
-      <c r="A96" s="16">
+      <c r="A96" s="15">
         <v>85</v>
       </c>
-      <c r="B96" s="14"/>
-      <c r="C96" s="14"/>
-      <c r="D96" s="14"/>
-      <c r="E96" s="14"/>
-      <c r="F96" s="14"/>
-      <c r="G96" s="7"/>
-      <c r="H96" s="13"/>
-      <c r="I96" s="12"/>
-      <c r="J96" s="13"/>
-      <c r="K96" s="12"/>
-      <c r="L96" s="12"/>
-      <c r="M96" s="12"/>
+      <c r="B96" s="13"/>
+      <c r="C96" s="13"/>
+      <c r="D96" s="13"/>
+      <c r="E96" s="13"/>
+      <c r="F96" s="13"/>
+      <c r="G96" s="6"/>
+      <c r="H96" s="12"/>
+      <c r="I96" s="11"/>
+      <c r="J96" s="12"/>
+      <c r="K96" s="11"/>
+      <c r="L96" s="11"/>
+      <c r="M96" s="11"/>
       <c r="N96" s="1"/>
       <c r="O96" s="1"/>
       <c r="P96" s="1"/>
@@ -5991,21 +5996,21 @@
       <c r="Z96" s="1"/>
     </row>
     <row r="97" spans="1:26" ht="15.75">
-      <c r="A97" s="18">
+      <c r="A97" s="17">
         <v>86</v>
       </c>
-      <c r="B97" s="15"/>
-      <c r="C97" s="15"/>
-      <c r="D97" s="15"/>
-      <c r="E97" s="15"/>
-      <c r="F97" s="15"/>
-      <c r="G97" s="8"/>
-      <c r="H97" s="15"/>
-      <c r="I97" s="10"/>
-      <c r="J97" s="15"/>
-      <c r="K97" s="10"/>
-      <c r="L97" s="9"/>
-      <c r="M97" s="9"/>
+      <c r="B97" s="14"/>
+      <c r="C97" s="14"/>
+      <c r="D97" s="14"/>
+      <c r="E97" s="14"/>
+      <c r="F97" s="14"/>
+      <c r="G97" s="7"/>
+      <c r="H97" s="14"/>
+      <c r="I97" s="9"/>
+      <c r="J97" s="14"/>
+      <c r="K97" s="9"/>
+      <c r="L97" s="8"/>
+      <c r="M97" s="8"/>
       <c r="N97" s="1"/>
       <c r="O97" s="1"/>
       <c r="P97" s="1"/>
@@ -6021,21 +6026,21 @@
       <c r="Z97" s="1"/>
     </row>
     <row r="98" spans="1:26" ht="15.75">
-      <c r="A98" s="16">
+      <c r="A98" s="15">
         <v>87</v>
       </c>
-      <c r="B98" s="14"/>
-      <c r="C98" s="14"/>
-      <c r="D98" s="14"/>
-      <c r="E98" s="14"/>
-      <c r="F98" s="14"/>
-      <c r="G98" s="7"/>
-      <c r="H98" s="13"/>
-      <c r="I98" s="12"/>
-      <c r="J98" s="13"/>
-      <c r="K98" s="12"/>
-      <c r="L98" s="12"/>
-      <c r="M98" s="12"/>
+      <c r="B98" s="13"/>
+      <c r="C98" s="13"/>
+      <c r="D98" s="13"/>
+      <c r="E98" s="13"/>
+      <c r="F98" s="13"/>
+      <c r="G98" s="6"/>
+      <c r="H98" s="12"/>
+      <c r="I98" s="11"/>
+      <c r="J98" s="12"/>
+      <c r="K98" s="11"/>
+      <c r="L98" s="11"/>
+      <c r="M98" s="11"/>
       <c r="N98" s="1"/>
       <c r="O98" s="1"/>
       <c r="P98" s="1"/>
@@ -6051,21 +6056,21 @@
       <c r="Z98" s="1"/>
     </row>
     <row r="99" spans="1:26" ht="15.75">
-      <c r="A99" s="18">
+      <c r="A99" s="17">
         <v>88</v>
       </c>
-      <c r="B99" s="15"/>
-      <c r="C99" s="15"/>
-      <c r="D99" s="15"/>
-      <c r="E99" s="15"/>
-      <c r="F99" s="15"/>
-      <c r="G99" s="8"/>
-      <c r="H99" s="15"/>
-      <c r="I99" s="10"/>
-      <c r="J99" s="15"/>
-      <c r="K99" s="10"/>
-      <c r="L99" s="9"/>
-      <c r="M99" s="9"/>
+      <c r="B99" s="14"/>
+      <c r="C99" s="14"/>
+      <c r="D99" s="14"/>
+      <c r="E99" s="14"/>
+      <c r="F99" s="14"/>
+      <c r="G99" s="7"/>
+      <c r="H99" s="14"/>
+      <c r="I99" s="9"/>
+      <c r="J99" s="14"/>
+      <c r="K99" s="9"/>
+      <c r="L99" s="8"/>
+      <c r="M99" s="8"/>
       <c r="N99" s="1"/>
       <c r="O99" s="1"/>
       <c r="P99" s="1"/>
@@ -6081,21 +6086,21 @@
       <c r="Z99" s="1"/>
     </row>
     <row r="100" spans="1:26" ht="15.75">
-      <c r="A100" s="16">
+      <c r="A100" s="15">
         <v>89</v>
       </c>
-      <c r="B100" s="14"/>
-      <c r="C100" s="14"/>
-      <c r="D100" s="14"/>
-      <c r="E100" s="14"/>
-      <c r="F100" s="14"/>
-      <c r="G100" s="7"/>
-      <c r="H100" s="13"/>
-      <c r="I100" s="12"/>
-      <c r="J100" s="13"/>
-      <c r="K100" s="12"/>
-      <c r="L100" s="12"/>
-      <c r="M100" s="12"/>
+      <c r="B100" s="13"/>
+      <c r="C100" s="13"/>
+      <c r="D100" s="13"/>
+      <c r="E100" s="13"/>
+      <c r="F100" s="13"/>
+      <c r="G100" s="6"/>
+      <c r="H100" s="12"/>
+      <c r="I100" s="11"/>
+      <c r="J100" s="12"/>
+      <c r="K100" s="11"/>
+      <c r="L100" s="11"/>
+      <c r="M100" s="11"/>
       <c r="N100" s="1"/>
       <c r="O100" s="1"/>
       <c r="P100" s="1"/>
@@ -6111,21 +6116,21 @@
       <c r="Z100" s="1"/>
     </row>
     <row r="101" spans="1:26" ht="15.75">
-      <c r="A101" s="18">
+      <c r="A101" s="17">
         <v>90</v>
       </c>
-      <c r="B101" s="15"/>
-      <c r="C101" s="15"/>
-      <c r="D101" s="15"/>
-      <c r="E101" s="15"/>
-      <c r="F101" s="15"/>
-      <c r="G101" s="8"/>
-      <c r="H101" s="15"/>
-      <c r="I101" s="10"/>
-      <c r="J101" s="15"/>
-      <c r="K101" s="10"/>
-      <c r="L101" s="9"/>
-      <c r="M101" s="9"/>
+      <c r="B101" s="14"/>
+      <c r="C101" s="14"/>
+      <c r="D101" s="14"/>
+      <c r="E101" s="14"/>
+      <c r="F101" s="14"/>
+      <c r="G101" s="7"/>
+      <c r="H101" s="14"/>
+      <c r="I101" s="9"/>
+      <c r="J101" s="14"/>
+      <c r="K101" s="9"/>
+      <c r="L101" s="8"/>
+      <c r="M101" s="8"/>
       <c r="N101" s="1"/>
       <c r="O101" s="1"/>
       <c r="P101" s="1"/>
@@ -6141,21 +6146,21 @@
       <c r="Z101" s="1"/>
     </row>
     <row r="102" spans="1:26" ht="15.75">
-      <c r="A102" s="16">
+      <c r="A102" s="15">
         <v>91</v>
       </c>
-      <c r="B102" s="14"/>
-      <c r="C102" s="14"/>
-      <c r="D102" s="14"/>
-      <c r="E102" s="14"/>
-      <c r="F102" s="14"/>
-      <c r="G102" s="7"/>
-      <c r="H102" s="13"/>
-      <c r="I102" s="12"/>
-      <c r="J102" s="13"/>
-      <c r="K102" s="12"/>
-      <c r="L102" s="12"/>
-      <c r="M102" s="12"/>
+      <c r="B102" s="13"/>
+      <c r="C102" s="13"/>
+      <c r="D102" s="13"/>
+      <c r="E102" s="13"/>
+      <c r="F102" s="13"/>
+      <c r="G102" s="6"/>
+      <c r="H102" s="12"/>
+      <c r="I102" s="11"/>
+      <c r="J102" s="12"/>
+      <c r="K102" s="11"/>
+      <c r="L102" s="11"/>
+      <c r="M102" s="11"/>
       <c r="N102" s="1"/>
       <c r="O102" s="1"/>
       <c r="P102" s="1"/>
@@ -6171,21 +6176,21 @@
       <c r="Z102" s="1"/>
     </row>
     <row r="103" spans="1:26" ht="15.75">
-      <c r="A103" s="18">
+      <c r="A103" s="17">
         <v>92</v>
       </c>
-      <c r="B103" s="15"/>
-      <c r="C103" s="15"/>
-      <c r="D103" s="15"/>
-      <c r="E103" s="15"/>
-      <c r="F103" s="15"/>
-      <c r="G103" s="8"/>
-      <c r="H103" s="15"/>
-      <c r="I103" s="10"/>
-      <c r="J103" s="15"/>
-      <c r="K103" s="10"/>
-      <c r="L103" s="9"/>
-      <c r="M103" s="9"/>
+      <c r="B103" s="14"/>
+      <c r="C103" s="14"/>
+      <c r="D103" s="14"/>
+      <c r="E103" s="14"/>
+      <c r="F103" s="14"/>
+      <c r="G103" s="7"/>
+      <c r="H103" s="14"/>
+      <c r="I103" s="9"/>
+      <c r="J103" s="14"/>
+      <c r="K103" s="9"/>
+      <c r="L103" s="8"/>
+      <c r="M103" s="8"/>
       <c r="N103" s="1"/>
       <c r="O103" s="1"/>
       <c r="P103" s="1"/>
@@ -6201,21 +6206,21 @@
       <c r="Z103" s="1"/>
     </row>
     <row r="104" spans="1:26" ht="15.75">
-      <c r="A104" s="16">
+      <c r="A104" s="15">
         <v>93</v>
       </c>
-      <c r="B104" s="14"/>
-      <c r="C104" s="14"/>
-      <c r="D104" s="14"/>
-      <c r="E104" s="14"/>
-      <c r="F104" s="14"/>
-      <c r="G104" s="7"/>
-      <c r="H104" s="13"/>
-      <c r="I104" s="12"/>
-      <c r="J104" s="13"/>
-      <c r="K104" s="12"/>
-      <c r="L104" s="12"/>
-      <c r="M104" s="12"/>
+      <c r="B104" s="13"/>
+      <c r="C104" s="13"/>
+      <c r="D104" s="13"/>
+      <c r="E104" s="13"/>
+      <c r="F104" s="13"/>
+      <c r="G104" s="6"/>
+      <c r="H104" s="12"/>
+      <c r="I104" s="11"/>
+      <c r="J104" s="12"/>
+      <c r="K104" s="11"/>
+      <c r="L104" s="11"/>
+      <c r="M104" s="11"/>
       <c r="N104" s="1"/>
       <c r="O104" s="1"/>
       <c r="P104" s="1"/>
@@ -6231,21 +6236,21 @@
       <c r="Z104" s="1"/>
     </row>
     <row r="105" spans="1:26" ht="15.75">
-      <c r="A105" s="18">
+      <c r="A105" s="17">
         <v>94</v>
       </c>
-      <c r="B105" s="15"/>
-      <c r="C105" s="15"/>
-      <c r="D105" s="15"/>
-      <c r="E105" s="15"/>
-      <c r="F105" s="15"/>
-      <c r="G105" s="8"/>
-      <c r="H105" s="15"/>
-      <c r="I105" s="10"/>
-      <c r="J105" s="15"/>
-      <c r="K105" s="10"/>
-      <c r="L105" s="9"/>
-      <c r="M105" s="9"/>
+      <c r="B105" s="14"/>
+      <c r="C105" s="14"/>
+      <c r="D105" s="14"/>
+      <c r="E105" s="14"/>
+      <c r="F105" s="14"/>
+      <c r="G105" s="7"/>
+      <c r="H105" s="14"/>
+      <c r="I105" s="9"/>
+      <c r="J105" s="14"/>
+      <c r="K105" s="9"/>
+      <c r="L105" s="8"/>
+      <c r="M105" s="8"/>
       <c r="N105" s="1"/>
       <c r="O105" s="1"/>
       <c r="P105" s="1"/>
@@ -6261,21 +6266,21 @@
       <c r="Z105" s="1"/>
     </row>
     <row r="106" spans="1:26" ht="15.75">
-      <c r="A106" s="16">
+      <c r="A106" s="15">
         <v>95</v>
       </c>
-      <c r="B106" s="14"/>
-      <c r="C106" s="14"/>
-      <c r="D106" s="14"/>
-      <c r="E106" s="14"/>
-      <c r="F106" s="14"/>
-      <c r="G106" s="7"/>
-      <c r="H106" s="13"/>
-      <c r="I106" s="12"/>
-      <c r="J106" s="13"/>
-      <c r="K106" s="12"/>
-      <c r="L106" s="12"/>
-      <c r="M106" s="12"/>
+      <c r="B106" s="13"/>
+      <c r="C106" s="13"/>
+      <c r="D106" s="13"/>
+      <c r="E106" s="13"/>
+      <c r="F106" s="13"/>
+      <c r="G106" s="6"/>
+      <c r="H106" s="12"/>
+      <c r="I106" s="11"/>
+      <c r="J106" s="12"/>
+      <c r="K106" s="11"/>
+      <c r="L106" s="11"/>
+      <c r="M106" s="11"/>
       <c r="N106" s="1"/>
       <c r="O106" s="1"/>
       <c r="P106" s="1"/>
@@ -6291,21 +6296,21 @@
       <c r="Z106" s="1"/>
     </row>
     <row r="107" spans="1:26" ht="15.75">
-      <c r="A107" s="18">
+      <c r="A107" s="17">
         <v>96</v>
       </c>
-      <c r="B107" s="15"/>
-      <c r="C107" s="15"/>
-      <c r="D107" s="15"/>
-      <c r="E107" s="15"/>
-      <c r="F107" s="15"/>
-      <c r="G107" s="8"/>
-      <c r="H107" s="15"/>
-      <c r="I107" s="10"/>
-      <c r="J107" s="15"/>
-      <c r="K107" s="10"/>
-      <c r="L107" s="9"/>
-      <c r="M107" s="9"/>
+      <c r="B107" s="14"/>
+      <c r="C107" s="14"/>
+      <c r="D107" s="14"/>
+      <c r="E107" s="14"/>
+      <c r="F107" s="14"/>
+      <c r="G107" s="7"/>
+      <c r="H107" s="14"/>
+      <c r="I107" s="9"/>
+      <c r="J107" s="14"/>
+      <c r="K107" s="9"/>
+      <c r="L107" s="8"/>
+      <c r="M107" s="8"/>
       <c r="N107" s="1"/>
       <c r="O107" s="1"/>
       <c r="P107" s="1"/>
@@ -6321,21 +6326,21 @@
       <c r="Z107" s="1"/>
     </row>
     <row r="108" spans="1:26" ht="15.75">
-      <c r="A108" s="16">
+      <c r="A108" s="15">
         <v>97</v>
       </c>
-      <c r="B108" s="14"/>
-      <c r="C108" s="14"/>
-      <c r="D108" s="14"/>
-      <c r="E108" s="14"/>
-      <c r="F108" s="14"/>
-      <c r="G108" s="7"/>
-      <c r="H108" s="13"/>
-      <c r="I108" s="12"/>
-      <c r="J108" s="13"/>
-      <c r="K108" s="12"/>
-      <c r="L108" s="12"/>
-      <c r="M108" s="12"/>
+      <c r="B108" s="13"/>
+      <c r="C108" s="13"/>
+      <c r="D108" s="13"/>
+      <c r="E108" s="13"/>
+      <c r="F108" s="13"/>
+      <c r="G108" s="6"/>
+      <c r="H108" s="12"/>
+      <c r="I108" s="11"/>
+      <c r="J108" s="12"/>
+      <c r="K108" s="11"/>
+      <c r="L108" s="11"/>
+      <c r="M108" s="11"/>
       <c r="N108" s="1"/>
       <c r="O108" s="1"/>
       <c r="P108" s="1"/>
@@ -6351,21 +6356,21 @@
       <c r="Z108" s="1"/>
     </row>
     <row r="109" spans="1:26" ht="15.75">
-      <c r="A109" s="18">
+      <c r="A109" s="17">
         <v>98</v>
       </c>
-      <c r="B109" s="15"/>
-      <c r="C109" s="15"/>
-      <c r="D109" s="15"/>
-      <c r="E109" s="15"/>
-      <c r="F109" s="15"/>
-      <c r="G109" s="8"/>
-      <c r="H109" s="15"/>
-      <c r="I109" s="10"/>
-      <c r="J109" s="15"/>
-      <c r="K109" s="10"/>
-      <c r="L109" s="9"/>
-      <c r="M109" s="9"/>
+      <c r="B109" s="14"/>
+      <c r="C109" s="14"/>
+      <c r="D109" s="14"/>
+      <c r="E109" s="14"/>
+      <c r="F109" s="14"/>
+      <c r="G109" s="7"/>
+      <c r="H109" s="14"/>
+      <c r="I109" s="9"/>
+      <c r="J109" s="14"/>
+      <c r="K109" s="9"/>
+      <c r="L109" s="8"/>
+      <c r="M109" s="8"/>
       <c r="N109" s="1"/>
       <c r="O109" s="1"/>
       <c r="P109" s="1"/>
@@ -6381,21 +6386,21 @@
       <c r="Z109" s="1"/>
     </row>
     <row r="110" spans="1:26" ht="15.75">
-      <c r="A110" s="16">
+      <c r="A110" s="15">
         <v>99</v>
       </c>
-      <c r="B110" s="14"/>
-      <c r="C110" s="14"/>
-      <c r="D110" s="14"/>
-      <c r="E110" s="14"/>
-      <c r="F110" s="14"/>
-      <c r="G110" s="7"/>
-      <c r="H110" s="13"/>
-      <c r="I110" s="12"/>
-      <c r="J110" s="13"/>
-      <c r="K110" s="12"/>
-      <c r="L110" s="12"/>
-      <c r="M110" s="12"/>
+      <c r="B110" s="13"/>
+      <c r="C110" s="13"/>
+      <c r="D110" s="13"/>
+      <c r="E110" s="13"/>
+      <c r="F110" s="13"/>
+      <c r="G110" s="6"/>
+      <c r="H110" s="12"/>
+      <c r="I110" s="11"/>
+      <c r="J110" s="12"/>
+      <c r="K110" s="11"/>
+      <c r="L110" s="11"/>
+      <c r="M110" s="11"/>
       <c r="N110" s="1"/>
       <c r="O110" s="1"/>
       <c r="P110" s="1"/>
@@ -6411,21 +6416,21 @@
       <c r="Z110" s="1"/>
     </row>
     <row r="111" spans="1:26" ht="15.75">
-      <c r="A111" s="18">
+      <c r="A111" s="17">
         <v>100</v>
       </c>
-      <c r="B111" s="15"/>
-      <c r="C111" s="15"/>
-      <c r="D111" s="15"/>
-      <c r="E111" s="15"/>
-      <c r="F111" s="15"/>
-      <c r="G111" s="8"/>
-      <c r="H111" s="15"/>
-      <c r="I111" s="10"/>
-      <c r="J111" s="15"/>
-      <c r="K111" s="10"/>
-      <c r="L111" s="9"/>
-      <c r="M111" s="9"/>
+      <c r="B111" s="14"/>
+      <c r="C111" s="14"/>
+      <c r="D111" s="14"/>
+      <c r="E111" s="14"/>
+      <c r="F111" s="14"/>
+      <c r="G111" s="7"/>
+      <c r="H111" s="14"/>
+      <c r="I111" s="9"/>
+      <c r="J111" s="14"/>
+      <c r="K111" s="9"/>
+      <c r="L111" s="8"/>
+      <c r="M111" s="8"/>
       <c r="N111" s="1"/>
       <c r="O111" s="1"/>
       <c r="P111" s="1"/>
@@ -6441,21 +6446,21 @@
       <c r="Z111" s="1"/>
     </row>
     <row r="112" spans="1:26" ht="15.75">
-      <c r="A112" s="16">
+      <c r="A112" s="15">
         <v>101</v>
       </c>
-      <c r="B112" s="14"/>
-      <c r="C112" s="14"/>
-      <c r="D112" s="14"/>
-      <c r="E112" s="14"/>
-      <c r="F112" s="14"/>
-      <c r="G112" s="7"/>
-      <c r="H112" s="13"/>
-      <c r="I112" s="12"/>
-      <c r="J112" s="13"/>
-      <c r="K112" s="12"/>
-      <c r="L112" s="12"/>
-      <c r="M112" s="12"/>
+      <c r="B112" s="13"/>
+      <c r="C112" s="13"/>
+      <c r="D112" s="13"/>
+      <c r="E112" s="13"/>
+      <c r="F112" s="13"/>
+      <c r="G112" s="6"/>
+      <c r="H112" s="12"/>
+      <c r="I112" s="11"/>
+      <c r="J112" s="12"/>
+      <c r="K112" s="11"/>
+      <c r="L112" s="11"/>
+      <c r="M112" s="11"/>
       <c r="N112" s="1"/>
       <c r="O112" s="1"/>
       <c r="P112" s="1"/>
@@ -6471,21 +6476,21 @@
       <c r="Z112" s="1"/>
     </row>
     <row r="113" spans="1:26" ht="15.75">
-      <c r="A113" s="18">
+      <c r="A113" s="17">
         <v>102</v>
       </c>
-      <c r="B113" s="15"/>
-      <c r="C113" s="15"/>
-      <c r="D113" s="15"/>
-      <c r="E113" s="15"/>
-      <c r="F113" s="15"/>
-      <c r="G113" s="8"/>
-      <c r="H113" s="15"/>
-      <c r="I113" s="10"/>
-      <c r="J113" s="15"/>
-      <c r="K113" s="10"/>
-      <c r="L113" s="9"/>
-      <c r="M113" s="9"/>
+      <c r="B113" s="14"/>
+      <c r="C113" s="14"/>
+      <c r="D113" s="14"/>
+      <c r="E113" s="14"/>
+      <c r="F113" s="14"/>
+      <c r="G113" s="7"/>
+      <c r="H113" s="14"/>
+      <c r="I113" s="9"/>
+      <c r="J113" s="14"/>
+      <c r="K113" s="9"/>
+      <c r="L113" s="8"/>
+      <c r="M113" s="8"/>
       <c r="N113" s="1"/>
       <c r="O113" s="1"/>
       <c r="P113" s="1"/>
@@ -6501,21 +6506,21 @@
       <c r="Z113" s="1"/>
     </row>
     <row r="114" spans="1:26" ht="15.75">
-      <c r="A114" s="16">
+      <c r="A114" s="15">
         <v>103</v>
       </c>
-      <c r="B114" s="14"/>
-      <c r="C114" s="14"/>
-      <c r="D114" s="14"/>
-      <c r="E114" s="14"/>
-      <c r="F114" s="14"/>
-      <c r="G114" s="7"/>
-      <c r="H114" s="13"/>
-      <c r="I114" s="12"/>
-      <c r="J114" s="13"/>
-      <c r="K114" s="12"/>
-      <c r="L114" s="12"/>
-      <c r="M114" s="12"/>
+      <c r="B114" s="13"/>
+      <c r="C114" s="13"/>
+      <c r="D114" s="13"/>
+      <c r="E114" s="13"/>
+      <c r="F114" s="13"/>
+      <c r="G114" s="6"/>
+      <c r="H114" s="12"/>
+      <c r="I114" s="11"/>
+      <c r="J114" s="12"/>
+      <c r="K114" s="11"/>
+      <c r="L114" s="11"/>
+      <c r="M114" s="11"/>
       <c r="N114" s="1"/>
       <c r="O114" s="1"/>
       <c r="P114" s="1"/>
@@ -6531,21 +6536,21 @@
       <c r="Z114" s="1"/>
     </row>
     <row r="115" spans="1:26" ht="15.75">
-      <c r="A115" s="18">
+      <c r="A115" s="17">
         <v>104</v>
       </c>
-      <c r="B115" s="15"/>
-      <c r="C115" s="15"/>
-      <c r="D115" s="15"/>
-      <c r="E115" s="15"/>
-      <c r="F115" s="15"/>
-      <c r="G115" s="8"/>
-      <c r="H115" s="15"/>
-      <c r="I115" s="10"/>
-      <c r="J115" s="15"/>
-      <c r="K115" s="10"/>
-      <c r="L115" s="9"/>
-      <c r="M115" s="9"/>
+      <c r="B115" s="14"/>
+      <c r="C115" s="14"/>
+      <c r="D115" s="14"/>
+      <c r="E115" s="14"/>
+      <c r="F115" s="14"/>
+      <c r="G115" s="7"/>
+      <c r="H115" s="14"/>
+      <c r="I115" s="9"/>
+      <c r="J115" s="14"/>
+      <c r="K115" s="9"/>
+      <c r="L115" s="8"/>
+      <c r="M115" s="8"/>
       <c r="N115" s="1"/>
       <c r="O115" s="1"/>
       <c r="P115" s="1"/>
@@ -6561,21 +6566,21 @@
       <c r="Z115" s="1"/>
     </row>
     <row r="116" spans="1:26" ht="15.75">
-      <c r="A116" s="16">
+      <c r="A116" s="15">
         <v>105</v>
       </c>
-      <c r="B116" s="14"/>
-      <c r="C116" s="14"/>
-      <c r="D116" s="14"/>
-      <c r="E116" s="14"/>
-      <c r="F116" s="14"/>
-      <c r="G116" s="7"/>
-      <c r="H116" s="13"/>
-      <c r="I116" s="12"/>
-      <c r="J116" s="13"/>
-      <c r="K116" s="12"/>
-      <c r="L116" s="12"/>
-      <c r="M116" s="12"/>
+      <c r="B116" s="13"/>
+      <c r="C116" s="13"/>
+      <c r="D116" s="13"/>
+      <c r="E116" s="13"/>
+      <c r="F116" s="13"/>
+      <c r="G116" s="6"/>
+      <c r="H116" s="12"/>
+      <c r="I116" s="11"/>
+      <c r="J116" s="12"/>
+      <c r="K116" s="11"/>
+      <c r="L116" s="11"/>
+      <c r="M116" s="11"/>
       <c r="N116" s="1"/>
       <c r="O116" s="1"/>
       <c r="P116" s="1"/>
@@ -6591,21 +6596,21 @@
       <c r="Z116" s="1"/>
     </row>
     <row r="117" spans="1:26" ht="15.75">
-      <c r="A117" s="18">
+      <c r="A117" s="17">
         <v>106</v>
       </c>
-      <c r="B117" s="15"/>
-      <c r="C117" s="15"/>
-      <c r="D117" s="15"/>
-      <c r="E117" s="15"/>
-      <c r="F117" s="15"/>
-      <c r="G117" s="8"/>
-      <c r="H117" s="15"/>
-      <c r="I117" s="10"/>
-      <c r="J117" s="15"/>
-      <c r="K117" s="10"/>
-      <c r="L117" s="9"/>
-      <c r="M117" s="9"/>
+      <c r="B117" s="14"/>
+      <c r="C117" s="14"/>
+      <c r="D117" s="14"/>
+      <c r="E117" s="14"/>
+      <c r="F117" s="14"/>
+      <c r="G117" s="7"/>
+      <c r="H117" s="14"/>
+      <c r="I117" s="9"/>
+      <c r="J117" s="14"/>
+      <c r="K117" s="9"/>
+      <c r="L117" s="8"/>
+      <c r="M117" s="8"/>
       <c r="N117" s="1"/>
       <c r="O117" s="1"/>
       <c r="P117" s="1"/>
@@ -6621,21 +6626,21 @@
       <c r="Z117" s="1"/>
     </row>
     <row r="118" spans="1:26" ht="15.75">
-      <c r="A118" s="16">
+      <c r="A118" s="15">
         <v>107</v>
       </c>
-      <c r="B118" s="14"/>
-      <c r="C118" s="14"/>
-      <c r="D118" s="14"/>
-      <c r="E118" s="14"/>
-      <c r="F118" s="14"/>
-      <c r="G118" s="7"/>
-      <c r="H118" s="13"/>
-      <c r="I118" s="12"/>
-      <c r="J118" s="13"/>
-      <c r="K118" s="12"/>
-      <c r="L118" s="12"/>
-      <c r="M118" s="12"/>
+      <c r="B118" s="13"/>
+      <c r="C118" s="13"/>
+      <c r="D118" s="13"/>
+      <c r="E118" s="13"/>
+      <c r="F118" s="13"/>
+      <c r="G118" s="6"/>
+      <c r="H118" s="12"/>
+      <c r="I118" s="11"/>
+      <c r="J118" s="12"/>
+      <c r="K118" s="11"/>
+      <c r="L118" s="11"/>
+      <c r="M118" s="11"/>
       <c r="N118" s="1"/>
       <c r="O118" s="1"/>
       <c r="P118" s="1"/>
@@ -6651,21 +6656,21 @@
       <c r="Z118" s="1"/>
     </row>
     <row r="119" spans="1:26" ht="15.75">
-      <c r="A119" s="18">
+      <c r="A119" s="17">
         <v>108</v>
       </c>
-      <c r="B119" s="15"/>
-      <c r="C119" s="15"/>
-      <c r="D119" s="15"/>
-      <c r="E119" s="15"/>
-      <c r="F119" s="15"/>
-      <c r="G119" s="8"/>
-      <c r="H119" s="15"/>
-      <c r="I119" s="10"/>
-      <c r="J119" s="15"/>
-      <c r="K119" s="10"/>
-      <c r="L119" s="9"/>
-      <c r="M119" s="9"/>
+      <c r="B119" s="14"/>
+      <c r="C119" s="14"/>
+      <c r="D119" s="14"/>
+      <c r="E119" s="14"/>
+      <c r="F119" s="14"/>
+      <c r="G119" s="7"/>
+      <c r="H119" s="14"/>
+      <c r="I119" s="9"/>
+      <c r="J119" s="14"/>
+      <c r="K119" s="9"/>
+      <c r="L119" s="8"/>
+      <c r="M119" s="8"/>
       <c r="N119" s="1"/>
       <c r="O119" s="1"/>
       <c r="P119" s="1"/>
@@ -8462,8 +8467,9 @@
   <hyperlinks>
     <hyperlink ref="E9" location="Werkwijze!A1" display="Uitleg over dit document vindt u in de tab &quot;werkwijze&quot; of klik hier" xr:uid="{76396179-941B-4D45-B955-A65BE48AA998}"/>
   </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" scale="55" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <drawing r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
@@ -8494,72 +8500,72 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:1">
-      <c r="A3" s="30" t="s">
+      <c r="A3" s="28" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" s="29"/>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" s="29" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
-      <c r="A4" s="31"/>
-    </row>
-    <row r="5" spans="1:1">
-      <c r="A5" s="31" t="s">
+    <row r="6" spans="1:1">
+      <c r="A6" s="29" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:1">
-      <c r="A6" s="31" t="s">
+    <row r="7" spans="1:1">
+      <c r="A7" s="29" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="7" spans="1:1">
-      <c r="A7" s="31" t="s">
+    <row r="8" spans="1:1">
+      <c r="A8" s="29"/>
+    </row>
+    <row r="11" spans="1:1">
+      <c r="A11" s="28" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:1">
-      <c r="A8" s="31"/>
-    </row>
-    <row r="11" spans="1:1">
-      <c r="A11" s="30" t="s">
+    <row r="12" spans="1:1">
+      <c r="A12" s="29"/>
+    </row>
+    <row r="13" spans="1:1">
+      <c r="A13" s="29" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:1">
-      <c r="A12" s="31"/>
-    </row>
-    <row r="13" spans="1:1">
-      <c r="A13" s="31" t="s">
+    <row r="14" spans="1:1">
+      <c r="A14" s="29" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="14" spans="1:1">
-      <c r="A14" s="31" t="s">
+    <row r="15" spans="1:1">
+      <c r="A15" s="29" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16" s="29" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17" s="29" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="15" spans="1:1">
-      <c r="A15" s="31" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1">
-      <c r="A16" s="31" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1">
-      <c r="A17" s="31" t="s">
-        <v>44</v>
-      </c>
-    </row>
     <row r="18" spans="1:1">
-      <c r="A18" s="31" t="s">
+      <c r="A18" s="29" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19" s="29" t="s">
         <v>35</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1">
-      <c r="A19" s="31" t="s">
-        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -8574,7 +8580,7 @@
   <sheetData>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -8605,18 +8611,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Omschrijving xmlns="fe46c194-0b3d-4916-a50a-1c7e6d47c726" xsi:nil="true"/>
-    <TaxCatchAll xmlns="765eb671-7931-41ea-bfdf-108cb9348ec6" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="fe46c194-0b3d-4916-a50a-1c7e6d47c726">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B7B24CEE30F9C741844B2BFCCED40860" ma:contentTypeVersion="15" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="e7cac4eec27caadbb4d440288f595866">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="fe46c194-0b3d-4916-a50a-1c7e6d47c726" xmlns:ns3="765eb671-7931-41ea-bfdf-108cb9348ec6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="45d053dfe2e6c2ea8f2bd42c76f4345c" ns2:_="" ns3:_="">
     <xsd:import namespace="fe46c194-0b3d-4916-a50a-1c7e6d47c726"/>
@@ -8851,14 +8845,26 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Omschrijving xmlns="fe46c194-0b3d-4916-a50a-1c7e6d47c726" xsi:nil="true"/>
+    <TaxCatchAll xmlns="765eb671-7931-41ea-bfdf-108cb9348ec6" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="fe46c194-0b3d-4916-a50a-1c7e6d47c726">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9181A8D5-F970-4B75-802F-42378AFD221B}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5BD4DFB8-481A-4C44-B158-5D5F4C3245A4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{92866CE2-4F20-4D4E-BB03-404CE375A9BC}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{92866CE2-4F20-4D4E-BB03-404CE375A9BC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5BD4DFB8-481A-4C44-B158-5D5F4C3245A4}"/>
 </file>
</xml_diff>